<commit_message>
Updated production data for Long Harbour
</commit_message>
<xml_diff>
--- a/data/Mappings/mapping_ghg.xlsx
+++ b/data/Mappings/mapping_ghg.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca-my.sharepoint.com/personal/marin_pellan_polymtl_ca/Documents/POST_DOC/CODE/metallican_db/data/Mappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="178" documentId="11_F25DC773A252ABDACC104887411C794C5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E67A0243-AFB4-423F-9499-DF45E76C2AC1}"/>
+  <xr:revisionPtr revIDLastSave="242" documentId="11_F25DC773A252ABDACC104887411C794C5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EECEBE50-B73F-461E-80AA-3FEA489169A1}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-705" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LT" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">LT!$A$1:$G$404</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">mapping!$A$1:$B$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">mapping!$A$1:$B$88</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1078" uniqueCount="683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="683">
   <si>
     <t>main_id</t>
   </si>
@@ -2546,7 +2546,7 @@
         <v>20.689655172413701</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>591</v>
       </c>
@@ -2569,7 +2569,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -2685,27 +2685,17 @@
       </c>
     </row>
     <row r="11" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="B11" s="2">
-        <v>10580</v>
-      </c>
-      <c r="C11" s="2">
-        <v>87.79</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="F11" s="2">
-        <v>50</v>
-      </c>
-      <c r="G11" s="2">
-        <v>18.518518518518501</v>
-      </c>
+      <c r="A11" t="s">
+        <v>395</v>
+      </c>
+      <c r="B11"/>
+      <c r="C11"/>
+      <c r="D11" t="s">
+        <v>396</v>
+      </c>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11"/>
     </row>
     <row r="12" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
@@ -2800,26 +2790,26 @@
       </c>
     </row>
     <row r="16" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="B16" s="2">
-        <v>10579</v>
-      </c>
-      <c r="C16" s="2">
-        <v>145.08000000000001</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="F16" s="2">
-        <v>100</v>
-      </c>
-      <c r="G16" s="2">
-        <v>100</v>
+      <c r="A16" t="s">
+        <v>580</v>
+      </c>
+      <c r="B16">
+        <v>12298</v>
+      </c>
+      <c r="C16">
+        <v>1937.93</v>
+      </c>
+      <c r="D16" t="s">
+        <v>581</v>
+      </c>
+      <c r="E16" t="s">
+        <v>658</v>
+      </c>
+      <c r="F16">
+        <v>35.294117647058798</v>
+      </c>
+      <c r="G16">
+        <v>16.6666666666666</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
@@ -3007,26 +2997,26 @@
       </c>
     </row>
     <row r="25" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
-        <v>586</v>
-      </c>
-      <c r="B25" s="2">
-        <v>12298</v>
-      </c>
-      <c r="C25" s="2">
-        <v>209.3</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>658</v>
-      </c>
-      <c r="F25" s="2">
-        <v>78.787878787878697</v>
-      </c>
-      <c r="G25" s="2">
-        <v>100</v>
+      <c r="A25" t="s">
+        <v>582</v>
+      </c>
+      <c r="B25">
+        <v>10580</v>
+      </c>
+      <c r="C25">
+        <v>393.62</v>
+      </c>
+      <c r="D25" t="s">
+        <v>583</v>
+      </c>
+      <c r="E25" t="s">
+        <v>259</v>
+      </c>
+      <c r="F25">
+        <v>44.4444444444444</v>
+      </c>
+      <c r="G25">
+        <v>15.6862745098039</v>
       </c>
     </row>
     <row r="26" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
@@ -3077,22 +3067,22 @@
     </row>
     <row r="28" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>598</v>
+        <v>586</v>
       </c>
       <c r="B28" s="2">
-        <v>10810</v>
+        <v>12298</v>
       </c>
       <c r="C28" s="2">
-        <v>229.35</v>
+        <v>209.3</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>599</v>
+        <v>585</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>600</v>
+        <v>658</v>
       </c>
       <c r="F28" s="2">
-        <v>100</v>
+        <v>78.787878787878697</v>
       </c>
       <c r="G28" s="2">
         <v>100</v>
@@ -3375,26 +3365,26 @@
       </c>
     </row>
     <row r="41" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>582</v>
-      </c>
-      <c r="B41">
-        <v>10580</v>
-      </c>
-      <c r="C41">
-        <v>393.62</v>
-      </c>
-      <c r="D41" t="s">
-        <v>583</v>
-      </c>
-      <c r="E41" t="s">
-        <v>259</v>
-      </c>
-      <c r="F41">
-        <v>44.4444444444444</v>
-      </c>
-      <c r="G41">
-        <v>15.6862745098039</v>
+      <c r="A41" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B41" s="2">
+        <v>12298</v>
+      </c>
+      <c r="C41" s="2">
+        <v>1756.27</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="F41" s="2">
+        <v>78.787878787878697</v>
+      </c>
+      <c r="G41" s="2">
+        <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
@@ -3421,26 +3411,26 @@
       </c>
     </row>
     <row r="43" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="B43" s="2">
+      <c r="A43" t="s">
+        <v>589</v>
+      </c>
+      <c r="B43">
         <v>10398</v>
       </c>
-      <c r="C43" s="2">
-        <v>402.62</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="E43" s="2" t="s">
+      <c r="C43">
+        <v>4225.47</v>
+      </c>
+      <c r="D43" t="s">
+        <v>590</v>
+      </c>
+      <c r="E43" t="s">
         <v>269</v>
       </c>
-      <c r="F43" s="2">
-        <v>100</v>
-      </c>
-      <c r="G43" s="2">
-        <v>100</v>
+      <c r="F43">
+        <v>50</v>
+      </c>
+      <c r="G43">
+        <v>16</v>
       </c>
     </row>
     <row r="44" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
@@ -3720,26 +3710,26 @@
       </c>
     </row>
     <row r="56" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="B56" s="2">
-        <v>10240</v>
-      </c>
-      <c r="C56" s="2">
-        <v>633.39</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="F56" s="2">
-        <v>100</v>
-      </c>
-      <c r="G56" s="2">
-        <v>100</v>
+      <c r="A56" t="s">
+        <v>589</v>
+      </c>
+      <c r="B56">
+        <v>12298</v>
+      </c>
+      <c r="C56">
+        <v>18361.259999999998</v>
+      </c>
+      <c r="D56" t="s">
+        <v>590</v>
+      </c>
+      <c r="E56" t="s">
+        <v>658</v>
+      </c>
+      <c r="F56">
+        <v>33.3333333333333</v>
+      </c>
+      <c r="G56">
+        <v>7.1428571428571299</v>
       </c>
     </row>
     <row r="57" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
@@ -3813,48 +3803,48 @@
     </row>
     <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
-        <v>593</v>
+        <v>262</v>
       </c>
       <c r="B60" s="2">
-        <v>10569</v>
+        <v>10579</v>
       </c>
       <c r="C60" s="2">
-        <v>736.22</v>
+        <v>145.08000000000001</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>594</v>
+        <v>263</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>595</v>
+        <v>264</v>
       </c>
       <c r="F60" s="2">
-        <v>64.285714285714207</v>
+        <v>100</v>
       </c>
       <c r="G60" s="2">
-        <v>59.259259259259203</v>
+        <v>100</v>
       </c>
     </row>
     <row r="61" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="B61" s="2">
-        <v>10570</v>
+        <v>10810</v>
       </c>
       <c r="C61" s="2">
-        <v>762.95</v>
+        <v>229.35</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="F61" s="2">
-        <v>91.6666666666666</v>
+        <v>100</v>
       </c>
       <c r="G61" s="2">
-        <v>64.705882352941103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="62" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
@@ -4041,7 +4031,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>31</v>
       </c>
@@ -4572,25 +4562,25 @@
     </row>
     <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>584</v>
+        <v>333</v>
       </c>
       <c r="B93">
-        <v>12298</v>
+        <v>10580</v>
       </c>
       <c r="C93">
-        <v>1756.27</v>
+        <v>5954.69</v>
       </c>
       <c r="D93" t="s">
-        <v>585</v>
+        <v>334</v>
       </c>
       <c r="E93" t="s">
-        <v>658</v>
+        <v>259</v>
       </c>
       <c r="F93">
-        <v>78.787878787878697</v>
+        <v>38.461538461538403</v>
       </c>
       <c r="G93">
-        <v>100</v>
+        <v>21.052631578947299</v>
       </c>
     </row>
     <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
@@ -4733,25 +4723,25 @@
     </row>
     <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>580</v>
+        <v>267</v>
       </c>
       <c r="B100">
-        <v>12298</v>
+        <v>10398</v>
       </c>
       <c r="C100">
-        <v>1937.93</v>
+        <v>9053.52</v>
       </c>
       <c r="D100" t="s">
-        <v>581</v>
+        <v>268</v>
       </c>
       <c r="E100" t="s">
-        <v>658</v>
+        <v>269</v>
       </c>
       <c r="F100">
-        <v>35.294117647058798</v>
+        <v>56.25</v>
       </c>
       <c r="G100">
-        <v>16.6666666666666</v>
+        <v>54.545454545454497</v>
       </c>
     </row>
     <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
@@ -5076,7 +5066,7 @@
         <v>19.672131147540899</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="4" t="s">
         <v>24</v>
       </c>
@@ -5214,7 +5204,7 @@
         <v>25.806451612903199</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>489</v>
       </c>
@@ -5329,7 +5319,7 @@
         <v>57.142857142857103</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>621</v>
       </c>
@@ -5354,25 +5344,10 @@
     </row>
     <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>589</v>
-      </c>
-      <c r="B127">
-        <v>10398</v>
-      </c>
-      <c r="C127">
-        <v>4225.47</v>
+        <v>148</v>
       </c>
       <c r="D127" t="s">
-        <v>590</v>
-      </c>
-      <c r="E127" t="s">
-        <v>269</v>
-      </c>
-      <c r="F127">
-        <v>50</v>
-      </c>
-      <c r="G127">
-        <v>16</v>
+        <v>149</v>
       </c>
     </row>
     <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
@@ -5584,25 +5559,10 @@
     </row>
     <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>333</v>
-      </c>
-      <c r="B137">
-        <v>10580</v>
-      </c>
-      <c r="C137">
-        <v>5954.69</v>
+        <v>136</v>
       </c>
       <c r="D137" t="s">
-        <v>334</v>
-      </c>
-      <c r="E137" t="s">
-        <v>259</v>
-      </c>
-      <c r="F137">
-        <v>38.461538461538403</v>
-      </c>
-      <c r="G137">
-        <v>21.052631578947299</v>
+        <v>137</v>
       </c>
     </row>
     <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
@@ -5789,7 +5749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>319</v>
       </c>
@@ -5905,26 +5865,26 @@
       </c>
     </row>
     <row r="151" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A151" t="s">
-        <v>267</v>
-      </c>
-      <c r="B151">
-        <v>10398</v>
-      </c>
-      <c r="C151">
-        <v>9053.52</v>
-      </c>
-      <c r="D151" t="s">
-        <v>268</v>
-      </c>
-      <c r="E151" t="s">
-        <v>269</v>
-      </c>
-      <c r="F151">
-        <v>56.25</v>
-      </c>
-      <c r="G151">
-        <v>54.545454545454497</v>
+      <c r="A151" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B151" s="2">
+        <v>10240</v>
+      </c>
+      <c r="C151" s="2">
+        <v>633.39</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="F151" s="2">
+        <v>100</v>
+      </c>
+      <c r="G151" s="2">
+        <v>100</v>
       </c>
     </row>
     <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
@@ -5996,7 +5956,7 @@
         <v>27.272727272727199</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>187</v>
       </c>
@@ -6594,7 +6554,7 @@
         <v>26.6666666666666</v>
       </c>
     </row>
-    <row r="181" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>576</v>
       </c>
@@ -7031,7 +6991,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>100</v>
       </c>
@@ -7285,26 +7245,26 @@
       </c>
     </row>
     <row r="211" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A211" t="s">
-        <v>589</v>
-      </c>
-      <c r="B211">
-        <v>12298</v>
-      </c>
-      <c r="C211">
-        <v>18361.259999999998</v>
-      </c>
-      <c r="D211" t="s">
-        <v>590</v>
-      </c>
-      <c r="E211" t="s">
-        <v>658</v>
-      </c>
-      <c r="F211">
-        <v>33.3333333333333</v>
-      </c>
-      <c r="G211">
-        <v>7.1428571428571299</v>
+      <c r="A211" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B211" s="2">
+        <v>10580</v>
+      </c>
+      <c r="C211" s="2">
+        <v>87.79</v>
+      </c>
+      <c r="D211" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="E211" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="F211" s="2">
+        <v>50</v>
+      </c>
+      <c r="G211" s="2">
+        <v>18.518518518518501</v>
       </c>
     </row>
     <row r="212" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
@@ -7330,7 +7290,7 @@
         <v>8.6956521739130395</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>345</v>
       </c>
@@ -7422,7 +7382,7 @@
         <v>14.285714285714199</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>15</v>
       </c>
@@ -7516,10 +7476,12 @@
       </c>
     </row>
     <row r="223" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A223" t="s">
+      <c r="A223" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D223" t="s">
+      <c r="B223" s="2"/>
+      <c r="C223" s="2"/>
+      <c r="D223" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -7531,7 +7493,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="225" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>38</v>
       </c>
@@ -7539,7 +7501,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="226" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>67</v>
       </c>
@@ -7547,7 +7509,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="227" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>69</v>
       </c>
@@ -7555,7 +7517,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="228" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>98</v>
       </c>
@@ -7563,7 +7525,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="229" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>106</v>
       </c>
@@ -7571,7 +7533,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="230" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>108</v>
       </c>
@@ -7579,7 +7541,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="231" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>110</v>
       </c>
@@ -7587,7 +7549,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="232" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>115</v>
       </c>
@@ -7595,7 +7557,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="233" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>117</v>
       </c>
@@ -7603,7 +7565,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="234" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>119</v>
       </c>
@@ -7611,7 +7573,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="235" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>123</v>
       </c>
@@ -7619,7 +7581,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="236" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>125</v>
       </c>
@@ -7627,15 +7589,30 @@
         <v>126</v>
       </c>
     </row>
-    <row r="237" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A237" t="s">
-        <v>136</v>
-      </c>
-      <c r="D237" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="238" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A237" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B237" s="2">
+        <v>10398</v>
+      </c>
+      <c r="C237" s="2">
+        <v>402.62</v>
+      </c>
+      <c r="D237" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="E237" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F237" s="2">
+        <v>100</v>
+      </c>
+      <c r="G237" s="2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>138</v>
       </c>
@@ -7643,7 +7620,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="239" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>140</v>
       </c>
@@ -7651,7 +7628,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="240" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>142</v>
       </c>
@@ -7659,7 +7636,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="241" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>144</v>
       </c>
@@ -7667,7 +7644,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="242" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>146</v>
       </c>
@@ -7675,15 +7652,30 @@
         <v>147</v>
       </c>
     </row>
-    <row r="243" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A243" t="s">
-        <v>148</v>
-      </c>
-      <c r="D243" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="244" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A243" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="B243" s="2">
+        <v>10569</v>
+      </c>
+      <c r="C243" s="2">
+        <v>736.22</v>
+      </c>
+      <c r="D243" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="E243" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="F243" s="2">
+        <v>64.285714285714207</v>
+      </c>
+      <c r="G243" s="2">
+        <v>59.259259259259203</v>
+      </c>
+    </row>
+    <row r="244" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>150</v>
       </c>
@@ -7691,7 +7683,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="245" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>152</v>
       </c>
@@ -7699,7 +7691,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="246" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>154</v>
       </c>
@@ -7707,7 +7699,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="247" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>158</v>
       </c>
@@ -7715,7 +7707,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="248" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>160</v>
       </c>
@@ -7723,7 +7715,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="249" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>162</v>
       </c>
@@ -7731,7 +7723,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="250" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>164</v>
       </c>
@@ -7739,7 +7731,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="251" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>166</v>
       </c>
@@ -7747,7 +7739,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="252" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>168</v>
       </c>
@@ -7755,7 +7747,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="253" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>176</v>
       </c>
@@ -7763,7 +7755,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="254" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>181</v>
       </c>
@@ -7771,7 +7763,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="255" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>183</v>
       </c>
@@ -7779,7 +7771,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="256" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>185</v>
       </c>
@@ -8171,7 +8163,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="305" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>378</v>
       </c>
@@ -8179,7 +8171,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="306" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>380</v>
       </c>
@@ -8187,7 +8179,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="307" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>382</v>
       </c>
@@ -8195,7 +8187,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="308" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>386</v>
       </c>
@@ -8203,7 +8195,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="309" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>388</v>
       </c>
@@ -8211,7 +8203,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="310" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>390</v>
       </c>
@@ -8219,15 +8211,30 @@
         <v>391</v>
       </c>
     </row>
-    <row r="311" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A311" t="s">
-        <v>395</v>
-      </c>
-      <c r="D311" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="312" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A311" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="B311" s="2">
+        <v>10570</v>
+      </c>
+      <c r="C311" s="2">
+        <v>762.95</v>
+      </c>
+      <c r="D311" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="E311" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F311" s="2">
+        <v>91.6666666666666</v>
+      </c>
+      <c r="G311" s="2">
+        <v>64.705882352941103</v>
+      </c>
+    </row>
+    <row r="312" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>400</v>
       </c>
@@ -8235,7 +8242,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="313" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>417</v>
       </c>
@@ -8243,7 +8250,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="314" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>420</v>
       </c>
@@ -8251,7 +8258,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="315" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
         <v>422</v>
       </c>
@@ -8259,7 +8266,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="316" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
         <v>424</v>
       </c>
@@ -8267,7 +8274,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="317" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
         <v>426</v>
       </c>
@@ -8275,7 +8282,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="318" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
         <v>428</v>
       </c>
@@ -8283,7 +8290,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="319" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
         <v>430</v>
       </c>
@@ -8291,7 +8298,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="320" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>432</v>
       </c>
@@ -8667,7 +8674,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B367">
         <v>10533</v>
       </c>
@@ -8691,7 +8698,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="370" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="370" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B370">
         <v>10658</v>
       </c>
@@ -8955,7 +8962,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="403" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="403" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B403">
         <v>11750</v>
       </c>
@@ -8975,14 +8982,7 @@
   <autoFilter ref="A1:G404" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="4">
       <filters>
-        <filter val="ARCELORMITTAL WINDSOR A DIVISION OF ARCELORMITTAL DOFASCO G.P"/>
-        <filter val="Division Goldex"/>
-        <filter val="Division Laronde"/>
-        <filter val="Division Meadowbank"/>
-        <filter val="North York Division"/>
-        <filter val="Patience Lake Division"/>
-        <filter val="Potash Corp - Allan Division"/>
-        <filter val="POTASH CORP - LANIGAN DIVISION"/>
+        <filter val="Port Colborne Refinery"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -8992,7 +8992,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A9FB282-8562-48BC-8F32-496757DDCE64}">
-  <dimension ref="A1:B266"/>
+  <dimension ref="A1:B263"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.54296875" bestFit="1" customWidth="1"/>
@@ -9622,10 +9622,10 @@
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A78">
+      <c r="A78" s="2">
         <v>12298</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="2" t="s">
         <v>586</v>
       </c>
     </row>
@@ -9701,203 +9701,211 @@
         <v>24</v>
       </c>
     </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A88">
+        <v>10863</v>
+      </c>
+      <c r="B88" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="225" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A225">
+        <v>10419</v>
+      </c>
+    </row>
+    <row r="226" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A226">
+        <v>10533</v>
+      </c>
+    </row>
+    <row r="227" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A227">
+        <v>10620</v>
+      </c>
+    </row>
     <row r="228" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A228">
-        <v>10419</v>
+        <v>10626</v>
       </c>
     </row>
     <row r="229" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A229">
-        <v>10533</v>
+        <v>10658</v>
       </c>
     </row>
     <row r="230" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A230">
-        <v>10620</v>
+        <v>10681</v>
       </c>
     </row>
     <row r="231" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A231">
-        <v>10626</v>
+        <v>10783</v>
       </c>
     </row>
     <row r="232" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A232">
-        <v>10658</v>
+        <v>10835</v>
       </c>
     </row>
     <row r="233" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A233">
-        <v>10681</v>
+        <v>10838</v>
       </c>
     </row>
     <row r="234" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A234">
-        <v>10783</v>
+        <v>10863</v>
       </c>
     </row>
     <row r="235" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A235">
-        <v>10835</v>
+        <v>10890</v>
       </c>
     </row>
     <row r="236" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A236">
-        <v>10838</v>
+        <v>10900</v>
       </c>
     </row>
     <row r="237" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A237">
-        <v>10863</v>
+        <v>10904</v>
       </c>
     </row>
     <row r="238" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A238">
-        <v>10890</v>
+        <v>10909</v>
       </c>
     </row>
     <row r="239" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A239">
-        <v>10900</v>
+        <v>10919</v>
       </c>
     </row>
     <row r="240" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A240">
-        <v>10904</v>
+        <v>10920</v>
       </c>
     </row>
     <row r="241" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A241">
-        <v>10909</v>
+        <v>10930</v>
       </c>
     </row>
     <row r="242" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A242">
-        <v>10919</v>
+        <v>11382</v>
       </c>
     </row>
     <row r="243" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A243">
-        <v>10920</v>
+        <v>11389</v>
       </c>
     </row>
     <row r="244" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A244">
-        <v>10930</v>
+        <v>11513</v>
       </c>
     </row>
     <row r="245" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A245">
-        <v>11382</v>
+        <v>11766</v>
       </c>
     </row>
     <row r="246" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A246">
-        <v>11389</v>
+        <v>11767</v>
       </c>
     </row>
     <row r="247" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A247">
-        <v>11513</v>
+        <v>11804</v>
       </c>
     </row>
     <row r="248" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A248">
-        <v>11766</v>
+        <v>11827</v>
       </c>
     </row>
     <row r="249" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A249">
-        <v>11767</v>
+        <v>11876</v>
       </c>
     </row>
     <row r="250" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A250">
-        <v>11804</v>
+        <v>11981</v>
       </c>
     </row>
     <row r="251" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A251">
-        <v>11827</v>
+        <v>12184</v>
       </c>
     </row>
     <row r="252" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A252">
-        <v>11876</v>
+        <v>12404</v>
       </c>
     </row>
     <row r="253" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A253">
-        <v>11981</v>
+        <v>12466</v>
       </c>
     </row>
     <row r="254" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A254">
-        <v>12184</v>
+        <v>12660</v>
       </c>
     </row>
     <row r="255" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A255">
-        <v>12404</v>
+        <v>12678</v>
       </c>
     </row>
     <row r="256" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A256">
-        <v>12466</v>
+        <v>12815</v>
       </c>
     </row>
     <row r="257" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A257">
-        <v>12660</v>
+        <v>12841</v>
       </c>
     </row>
     <row r="258" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A258">
-        <v>12678</v>
+        <v>10306</v>
       </c>
     </row>
     <row r="259" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A259">
-        <v>12815</v>
+        <v>10647</v>
       </c>
     </row>
     <row r="260" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A260">
-        <v>12841</v>
+        <v>11046</v>
       </c>
     </row>
     <row r="261" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A261">
-        <v>10306</v>
+        <v>11103</v>
       </c>
     </row>
     <row r="262" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A262">
-        <v>10647</v>
+        <v>11750</v>
       </c>
     </row>
     <row r="263" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A263">
-        <v>11046</v>
-      </c>
-    </row>
-    <row r="264" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A264">
-        <v>11103</v>
-      </c>
-    </row>
-    <row r="265" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A265">
-        <v>11750</v>
-      </c>
-    </row>
-    <row r="266" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A266">
         <v>12555</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B87" xr:uid="{9A9FB282-8562-48BC-8F32-496757DDCE64}"/>
+  <autoFilter ref="A1:B88" xr:uid="{9A9FB282-8562-48BC-8F32-496757DDCE64}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added carbon stock ecosystems table
</commit_message>
<xml_diff>
--- a/data/Mappings/mapping_ghg.xlsx
+++ b/data/Mappings/mapping_ghg.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca-my.sharepoint.com/personal/marin_pellan_polymtl_ca/Documents/POST_DOC/CODE/metallican_db/data/Mappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="279" documentId="11_F25DC773A252ABDACC104887411C794C5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B8F2A6B-B7F5-417E-8E36-4C6C8A7D94F9}"/>
+  <xr:revisionPtr revIDLastSave="321" documentId="11_F25DC773A252ABDACC104887411C794C5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B593DDF9-079C-45D5-A9CC-91D11B21CCBA}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LT" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">LT!$A$1:$G$404</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">mapping!$A$1:$B$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">mapping!$A$1:$B$91</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="683">
   <si>
     <t>main_id</t>
   </si>
@@ -2448,19 +2448,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G404"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="62.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="62.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2483,7 +2484,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>191</v>
       </c>
@@ -2506,7 +2507,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>359</v>
       </c>
@@ -2529,7 +2530,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>576</v>
       </c>
@@ -2552,7 +2553,7 @@
         <v>20.689655172413701</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>591</v>
       </c>
@@ -2575,7 +2576,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -2598,7 +2599,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>361</v>
       </c>
@@ -2621,7 +2622,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>463</v>
       </c>
@@ -2644,7 +2645,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>85</v>
       </c>
@@ -2667,21 +2668,21 @@
         <v>54.545454545454497</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>127</v>
+        <v>442</v>
       </c>
       <c r="B10" s="2">
-        <v>10923</v>
+        <v>10908</v>
       </c>
       <c r="C10" s="2">
-        <v>77.88</v>
+        <v>11516.07</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>128</v>
+        <v>443</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>129</v>
+        <v>180</v>
       </c>
       <c r="F10" s="2">
         <v>100</v>
@@ -2690,7 +2691,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>395</v>
       </c>
@@ -2703,7 +2704,7 @@
       <c r="F11"/>
       <c r="G11"/>
     </row>
-    <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>324</v>
       </c>
@@ -2726,7 +2727,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>255</v>
       </c>
@@ -2749,7 +2750,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>453</v>
       </c>
@@ -2772,7 +2773,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>539</v>
       </c>
@@ -2795,7 +2796,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>580</v>
       </c>
@@ -2818,7 +2819,7 @@
         <v>16.6666666666666</v>
       </c>
     </row>
-    <row r="17" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>467</v>
       </c>
@@ -2841,7 +2842,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>48</v>
       </c>
@@ -2864,7 +2865,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>298</v>
       </c>
@@ -2887,7 +2888,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>477</v>
       </c>
@@ -2910,7 +2911,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>465</v>
       </c>
@@ -2933,7 +2934,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="22" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>202</v>
       </c>
@@ -2956,7 +2957,7 @@
         <v>58.823529411764703</v>
       </c>
     </row>
-    <row r="23" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>547</v>
       </c>
@@ -2979,7 +2980,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>552</v>
       </c>
@@ -3002,7 +3003,7 @@
         <v>37.5</v>
       </c>
     </row>
-    <row r="25" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>582</v>
       </c>
@@ -3025,7 +3026,7 @@
         <v>15.6862745098039</v>
       </c>
     </row>
-    <row r="26" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>43</v>
       </c>
@@ -3048,7 +3049,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>502</v>
       </c>
@@ -3071,7 +3072,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="28" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>586</v>
       </c>
@@ -3094,7 +3095,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="29" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>85</v>
       </c>
@@ -3117,7 +3118,7 @@
         <v>56.521739130434703</v>
       </c>
     </row>
-    <row r="30" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>250</v>
       </c>
@@ -3140,7 +3141,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="31" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>63</v>
       </c>
@@ -3163,7 +3164,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>112</v>
       </c>
@@ -3186,7 +3187,7 @@
         <v>55.172413793103402</v>
       </c>
     </row>
-    <row r="33" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>59</v>
       </c>
@@ -3209,7 +3210,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>15</v>
       </c>
@@ -3232,7 +3233,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>45</v>
       </c>
@@ -3255,7 +3256,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>245</v>
       </c>
@@ -3278,7 +3279,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="37" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>562</v>
       </c>
@@ -3301,7 +3302,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="38" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>412</v>
       </c>
@@ -3324,7 +3325,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="39" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>448</v>
       </c>
@@ -3347,7 +3348,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>402</v>
       </c>
@@ -3370,7 +3371,7 @@
         <v>23.529411764705799</v>
       </c>
     </row>
-    <row r="41" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>584</v>
       </c>
@@ -3393,7 +3394,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="42" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>465</v>
       </c>
@@ -3416,7 +3417,7 @@
         <v>18.518518518518501</v>
       </c>
     </row>
-    <row r="43" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>589</v>
       </c>
@@ -3439,7 +3440,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="44" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>479</v>
       </c>
@@ -3462,7 +3463,7 @@
         <v>34.567901234567898</v>
       </c>
     </row>
-    <row r="45" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>474</v>
       </c>
@@ -3485,7 +3486,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>74</v>
       </c>
@@ -3508,7 +3509,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="47" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>252</v>
       </c>
@@ -3531,7 +3532,7 @@
         <v>15.0537634408602</v>
       </c>
     </row>
-    <row r="48" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>87</v>
       </c>
@@ -3554,7 +3555,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="49" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>121</v>
       </c>
@@ -3577,7 +3578,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="50" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>199</v>
       </c>
@@ -3600,7 +3601,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="51" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>456</v>
       </c>
@@ -3623,7 +3624,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>470</v>
       </c>
@@ -3646,7 +3647,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>248</v>
       </c>
@@ -3669,7 +3670,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="54" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>450</v>
       </c>
@@ -3692,7 +3693,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>460</v>
       </c>
@@ -3715,7 +3716,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="56" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>589</v>
       </c>
@@ -3738,7 +3739,7 @@
         <v>7.1428571428571299</v>
       </c>
     </row>
-    <row r="57" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>241</v>
       </c>
@@ -3761,7 +3762,7 @@
         <v>57.142857142857103</v>
       </c>
     </row>
-    <row r="58" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>456</v>
       </c>
@@ -3784,7 +3785,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="59" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>456</v>
       </c>
@@ -3807,7 +3808,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>262</v>
       </c>
@@ -3830,7 +3831,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="61" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>598</v>
       </c>
@@ -3853,7 +3854,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="62" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>51</v>
       </c>
@@ -3876,7 +3877,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="63" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>238</v>
       </c>
@@ -3899,7 +3900,7 @@
         <v>26.6666666666666</v>
       </c>
     </row>
-    <row r="64" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>321</v>
       </c>
@@ -3922,7 +3923,7 @@
         <v>33.3333333333333</v>
       </c>
     </row>
-    <row r="65" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>28</v>
       </c>
@@ -3945,7 +3946,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="66" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>19</v>
       </c>
@@ -3968,7 +3969,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="67" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>522</v>
       </c>
@@ -3991,7 +3992,7 @@
         <v>20.8333333333333</v>
       </c>
     </row>
-    <row r="68" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>409</v>
       </c>
@@ -4014,7 +4015,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>537</v>
       </c>
@@ -4037,7 +4038,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>31</v>
       </c>
@@ -4060,7 +4061,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="71" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>63</v>
       </c>
@@ -4083,7 +4084,7 @@
         <v>66.6666666666666</v>
       </c>
     </row>
-    <row r="72" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>77</v>
       </c>
@@ -4106,7 +4107,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="73" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>465</v>
       </c>
@@ -4129,7 +4130,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>170</v>
       </c>
@@ -4152,7 +4153,7 @@
         <v>33.3333333333333</v>
       </c>
     </row>
-    <row r="75" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>59</v>
       </c>
@@ -4175,21 +4176,21 @@
         <v>23.076923076922998</v>
       </c>
     </row>
-    <row r="76" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2">
-        <v>10922</v>
+        <v>10923</v>
       </c>
       <c r="C76" s="2">
-        <v>1125.68</v>
+        <v>77.88</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="F76" s="2">
         <v>100</v>
@@ -4198,7 +4199,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="77" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>566</v>
       </c>
@@ -4221,7 +4222,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="78" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>524</v>
       </c>
@@ -4244,7 +4245,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>90</v>
       </c>
@@ -4267,7 +4268,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>541</v>
       </c>
@@ -4290,7 +4291,7 @@
         <v>55.172413793103402</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>257</v>
       </c>
@@ -4313,7 +4314,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="82" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>196</v>
       </c>
@@ -4336,7 +4337,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>51</v>
       </c>
@@ -4359,7 +4360,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>522</v>
       </c>
@@ -4382,7 +4383,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>522</v>
       </c>
@@ -4405,7 +4406,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>51</v>
       </c>
@@ -4428,7 +4429,7 @@
         <v>7.8431372549019596</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>90</v>
       </c>
@@ -4451,7 +4452,7 @@
         <v>29.090909090909001</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>202</v>
       </c>
@@ -4474,7 +4475,7 @@
         <v>48.8888888888888</v>
       </c>
     </row>
-    <row r="89" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>495</v>
       </c>
@@ -4497,7 +4498,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>527</v>
       </c>
@@ -4520,7 +4521,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>319</v>
       </c>
@@ -4543,7 +4544,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>174</v>
       </c>
@@ -4566,7 +4567,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>333</v>
       </c>
@@ -4589,7 +4590,7 @@
         <v>21.052631578947299</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>319</v>
       </c>
@@ -4612,7 +4613,7 @@
         <v>37.037037037037003</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>90</v>
       </c>
@@ -4635,7 +4636,7 @@
         <v>76.470588235294102</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>392</v>
       </c>
@@ -4658,7 +4659,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="97" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>606</v>
       </c>
@@ -4681,7 +4682,7 @@
         <v>51.428571428571402</v>
       </c>
     </row>
-    <row r="98" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>522</v>
       </c>
@@ -4704,7 +4705,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>90</v>
       </c>
@@ -4727,7 +4728,7 @@
         <v>20.689655172413701</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>267</v>
       </c>
@@ -4750,7 +4751,7 @@
         <v>54.545454545454497</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>130</v>
       </c>
@@ -4773,7 +4774,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>90</v>
       </c>
@@ -4796,7 +4797,7 @@
         <v>23.8095238095238</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>519</v>
       </c>
@@ -4819,7 +4820,7 @@
         <v>27.7777777777777</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>397</v>
       </c>
@@ -4842,7 +4843,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>156</v>
       </c>
@@ -4865,7 +4866,7 @@
         <v>66.6666666666666</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>623</v>
       </c>
@@ -4888,7 +4889,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>81</v>
       </c>
@@ -4911,7 +4912,7 @@
         <v>59.090909090909001</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>302</v>
       </c>
@@ -4934,7 +4935,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>81</v>
       </c>
@@ -4957,7 +4958,7 @@
         <v>52.173913043478201</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>557</v>
       </c>
@@ -4980,7 +4981,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>191</v>
       </c>
@@ -5003,7 +5004,7 @@
         <v>21.428571428571399</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>465</v>
       </c>
@@ -5026,7 +5027,7 @@
         <v>19.354838709677399</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>406</v>
       </c>
@@ -5049,7 +5050,7 @@
         <v>12.1212121212121</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>191</v>
       </c>
@@ -5072,7 +5073,7 @@
         <v>19.672131147540899</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="4" t="s">
         <v>24</v>
       </c>
@@ -5095,7 +5096,7 @@
         <v>52.173913043478201</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>414</v>
       </c>
@@ -5118,7 +5119,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>300</v>
       </c>
@@ -5141,7 +5142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>522</v>
       </c>
@@ -5164,7 +5165,7 @@
         <v>72.727272727272705</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>456</v>
       </c>
@@ -5187,7 +5188,7 @@
         <v>14.285714285714199</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>191</v>
       </c>
@@ -5210,7 +5211,7 @@
         <v>25.806451612903199</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>489</v>
       </c>
@@ -5233,7 +5234,7 @@
         <v>30.769230769230699</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>576</v>
       </c>
@@ -5256,7 +5257,7 @@
         <v>34.285714285714199</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>71</v>
       </c>
@@ -5279,7 +5280,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>51</v>
       </c>
@@ -5302,7 +5303,7 @@
         <v>14.285714285714199</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>305</v>
       </c>
@@ -5325,7 +5326,7 @@
         <v>57.142857142857103</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>621</v>
       </c>
@@ -5348,7 +5349,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>148</v>
       </c>
@@ -5356,7 +5357,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>541</v>
       </c>
@@ -5379,7 +5380,7 @@
         <v>40.909090909090899</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>100</v>
       </c>
@@ -5402,7 +5403,7 @@
         <v>6.6666666666666696</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>406</v>
       </c>
@@ -5425,7 +5426,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>402</v>
       </c>
@@ -5448,7 +5449,7 @@
         <v>41.379310344827502</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>194</v>
       </c>
@@ -5471,7 +5472,7 @@
         <v>31.25</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>384</v>
       </c>
@@ -5494,7 +5495,7 @@
         <v>23.076923076922998</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>539</v>
       </c>
@@ -5517,7 +5518,7 @@
         <v>10.5263157894736</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>270</v>
       </c>
@@ -5540,7 +5541,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>412</v>
       </c>
@@ -5563,7 +5564,7 @@
         <v>17.647058823529399</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>136</v>
       </c>
@@ -5571,7 +5572,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>194</v>
       </c>
@@ -5594,7 +5595,7 @@
         <v>46.511627906976699</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>384</v>
       </c>
@@ -5617,7 +5618,7 @@
         <v>31.746031746031701</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>448</v>
       </c>
@@ -5640,7 +5641,7 @@
         <v>30.303030303030202</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>24</v>
       </c>
@@ -5663,7 +5664,7 @@
         <v>42.857142857142797</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>24</v>
       </c>
@@ -5686,7 +5687,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>170</v>
       </c>
@@ -5709,7 +5710,7 @@
         <v>20.8333333333333</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>100</v>
       </c>
@@ -5732,7 +5733,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>255</v>
       </c>
@@ -5755,7 +5756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>319</v>
       </c>
@@ -5778,7 +5779,7 @@
         <v>26.6666666666666</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>307</v>
       </c>
@@ -5801,7 +5802,7 @@
         <v>23.529411764705799</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>100</v>
       </c>
@@ -5824,7 +5825,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>156</v>
       </c>
@@ -5847,7 +5848,7 @@
         <v>20.689655172413701</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>498</v>
       </c>
@@ -5870,7 +5871,7 @@
         <v>9.0909090909090899</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>272</v>
       </c>
@@ -5893,7 +5894,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>347</v>
       </c>
@@ -5916,7 +5917,7 @@
         <v>25.6410256410256</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>329</v>
       </c>
@@ -5939,7 +5940,7 @@
         <v>66.6666666666666</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>96</v>
       </c>
@@ -5962,7 +5963,7 @@
         <v>27.272727272727199</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>187</v>
       </c>
@@ -5985,7 +5986,7 @@
         <v>9.0909090909090899</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>587</v>
       </c>
@@ -6008,7 +6009,7 @@
         <v>23.728813559321999</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>591</v>
       </c>
@@ -6031,7 +6032,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>234</v>
       </c>
@@ -6054,7 +6055,7 @@
         <v>27.118644067796598</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>40</v>
       </c>
@@ -6077,7 +6078,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>359</v>
       </c>
@@ -6100,7 +6101,7 @@
         <v>26.229508196721302</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>412</v>
       </c>
@@ -6123,7 +6124,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>361</v>
       </c>
@@ -6146,7 +6147,7 @@
         <v>11.764705882352899</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>51</v>
       </c>
@@ -6169,7 +6170,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>448</v>
       </c>
@@ -6192,7 +6193,7 @@
         <v>26.6666666666666</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>456</v>
       </c>
@@ -6215,7 +6216,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="5" t="s">
         <v>311</v>
       </c>
@@ -6238,21 +6239,21 @@
         <v>57.142857142857103</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>442</v>
+        <v>133</v>
       </c>
       <c r="B167" s="2">
-        <v>10908</v>
+        <v>10922</v>
       </c>
       <c r="C167" s="2">
-        <v>11516.07</v>
+        <v>1125.68</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>443</v>
+        <v>134</v>
       </c>
       <c r="E167" s="2" t="s">
-        <v>180</v>
+        <v>135</v>
       </c>
       <c r="F167" s="2">
         <v>100</v>
@@ -6261,7 +6262,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>465</v>
       </c>
@@ -6284,7 +6285,7 @@
         <v>26.086956521739101</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>359</v>
       </c>
@@ -6307,7 +6308,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>77</v>
       </c>
@@ -6330,7 +6331,7 @@
         <v>14.285714285714199</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>361</v>
       </c>
@@ -6353,7 +6354,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>359</v>
       </c>
@@ -6376,7 +6377,7 @@
         <v>32.258064516128997</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>361</v>
       </c>
@@ -6399,7 +6400,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>625</v>
       </c>
@@ -6422,7 +6423,7 @@
         <v>17.7777777777777</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>463</v>
       </c>
@@ -6445,7 +6446,7 @@
         <v>18.75</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>178</v>
       </c>
@@ -6468,7 +6469,7 @@
         <v>18.75</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>241</v>
       </c>
@@ -6491,7 +6492,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>191</v>
       </c>
@@ -6514,7 +6515,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>250</v>
       </c>
@@ -6537,7 +6538,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>591</v>
       </c>
@@ -6560,7 +6561,7 @@
         <v>26.6666666666666</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>576</v>
       </c>
@@ -6583,7 +6584,7 @@
         <v>23.529411764705799</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>359</v>
       </c>
@@ -6606,7 +6607,7 @@
         <v>26.315789473684202</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>191</v>
       </c>
@@ -6629,7 +6630,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>361</v>
       </c>
@@ -6652,7 +6653,7 @@
         <v>21.428571428571399</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>448</v>
       </c>
@@ -6675,7 +6676,7 @@
         <v>11.4285714285714</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>402</v>
       </c>
@@ -6698,7 +6699,7 @@
         <v>29.629629629629601</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
         <v>619</v>
       </c>
@@ -6721,7 +6722,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>463</v>
       </c>
@@ -6744,7 +6745,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>463</v>
       </c>
@@ -6767,7 +6768,7 @@
         <v>27.272727272727199</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
         <v>406</v>
       </c>
@@ -6790,7 +6791,7 @@
         <v>46.6666666666666</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>465</v>
       </c>
@@ -6813,7 +6814,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>329</v>
       </c>
@@ -6836,7 +6837,7 @@
         <v>19.354838709677399</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>456</v>
       </c>
@@ -6859,7 +6860,7 @@
         <v>18.181818181818102</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>463</v>
       </c>
@@ -6882,7 +6883,7 @@
         <v>21.818181818181799</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>574</v>
       </c>
@@ -6905,7 +6906,7 @@
         <v>26.315789473684202</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>51</v>
       </c>
@@ -6928,7 +6929,7 @@
         <v>18.181818181818102</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>458</v>
       </c>
@@ -6951,7 +6952,7 @@
         <v>29.629629629629601</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>535</v>
       </c>
@@ -6974,7 +6975,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>621</v>
       </c>
@@ -6997,7 +6998,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>100</v>
       </c>
@@ -7020,7 +7021,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>412</v>
       </c>
@@ -7043,7 +7044,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>347</v>
       </c>
@@ -7066,7 +7067,7 @@
         <v>24.5614035087719</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>5</v>
       </c>
@@ -7089,7 +7090,7 @@
         <v>27.7777777777777</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>234</v>
       </c>
@@ -7112,7 +7113,7 @@
         <v>16.326530612244799</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>234</v>
       </c>
@@ -7135,7 +7136,7 @@
         <v>4.6511627906976596</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>489</v>
       </c>
@@ -7158,7 +7159,7 @@
         <v>5.8823529411764603</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>406</v>
       </c>
@@ -7181,7 +7182,7 @@
         <v>22.857142857142801</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>234</v>
       </c>
@@ -7204,7 +7205,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>347</v>
       </c>
@@ -7227,7 +7228,7 @@
         <v>20.689655172413701</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>48</v>
       </c>
@@ -7250,7 +7251,7 @@
         <v>15.3846153846153</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>276</v>
       </c>
@@ -7273,7 +7274,7 @@
         <v>18.518518518518501</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>347</v>
       </c>
@@ -7296,7 +7297,7 @@
         <v>8.6956521739130395</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>345</v>
       </c>
@@ -7319,7 +7320,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>458</v>
       </c>
@@ -7342,7 +7343,7 @@
         <v>12.1212121212121</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>294</v>
       </c>
@@ -7365,7 +7366,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>22</v>
       </c>
@@ -7388,7 +7389,7 @@
         <v>14.285714285714199</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>15</v>
       </c>
@@ -7411,7 +7412,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>402</v>
       </c>
@@ -7434,7 +7435,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
         <v>450</v>
       </c>
@@ -7457,7 +7458,7 @@
         <v>73.684210526315795</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>8</v>
       </c>
@@ -7465,7 +7466,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>10</v>
       </c>
@@ -7473,7 +7474,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>13</v>
       </c>
@@ -7481,7 +7482,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
         <v>34</v>
       </c>
@@ -7491,7 +7492,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>36</v>
       </c>
@@ -7499,7 +7500,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>38</v>
       </c>
@@ -7507,7 +7508,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>67</v>
       </c>
@@ -7515,7 +7516,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>69</v>
       </c>
@@ -7523,7 +7524,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>98</v>
       </c>
@@ -7531,7 +7532,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>106</v>
       </c>
@@ -7539,7 +7540,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>108</v>
       </c>
@@ -7547,7 +7548,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>110</v>
       </c>
@@ -7555,7 +7556,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>115</v>
       </c>
@@ -7563,7 +7564,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>117</v>
       </c>
@@ -7571,7 +7572,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>119</v>
       </c>
@@ -7579,7 +7580,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>123</v>
       </c>
@@ -7587,7 +7588,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>125</v>
       </c>
@@ -7595,7 +7596,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A237" s="2" t="s">
         <v>278</v>
       </c>
@@ -7618,7 +7619,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>138</v>
       </c>
@@ -7626,7 +7627,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>140</v>
       </c>
@@ -7634,7 +7635,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>142</v>
       </c>
@@ -7642,7 +7643,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>144</v>
       </c>
@@ -7650,7 +7651,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>146</v>
       </c>
@@ -7658,7 +7659,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A243" s="2" t="s">
         <v>593</v>
       </c>
@@ -7681,7 +7682,7 @@
         <v>59.259259259259203</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>150</v>
       </c>
@@ -7689,7 +7690,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>152</v>
       </c>
@@ -7697,7 +7698,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>154</v>
       </c>
@@ -7705,7 +7706,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>158</v>
       </c>
@@ -7713,7 +7714,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>160</v>
       </c>
@@ -7721,7 +7722,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>162</v>
       </c>
@@ -7729,7 +7730,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>164</v>
       </c>
@@ -7737,7 +7738,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>166</v>
       </c>
@@ -7745,7 +7746,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>168</v>
       </c>
@@ -7753,7 +7754,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>176</v>
       </c>
@@ -7761,7 +7762,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>181</v>
       </c>
@@ -7769,7 +7770,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>183</v>
       </c>
@@ -7777,7 +7778,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>185</v>
       </c>
@@ -7785,7 +7786,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="257" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>189</v>
       </c>
@@ -7793,7 +7794,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="258" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>204</v>
       </c>
@@ -7801,7 +7802,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="259" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>206</v>
       </c>
@@ -7809,7 +7810,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="260" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>208</v>
       </c>
@@ -7817,7 +7818,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="261" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>210</v>
       </c>
@@ -7825,7 +7826,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="262" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>212</v>
       </c>
@@ -7833,7 +7834,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="263" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>214</v>
       </c>
@@ -7841,7 +7842,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="264" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>216</v>
       </c>
@@ -7849,7 +7850,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="265" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>218</v>
       </c>
@@ -7857,7 +7858,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="266" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>220</v>
       </c>
@@ -7865,7 +7866,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="267" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>222</v>
       </c>
@@ -7873,7 +7874,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="268" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>224</v>
       </c>
@@ -7881,7 +7882,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="269" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>226</v>
       </c>
@@ -7889,7 +7890,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="270" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>228</v>
       </c>
@@ -7897,7 +7898,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="271" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>230</v>
       </c>
@@ -7905,7 +7906,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="272" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>232</v>
       </c>
@@ -7913,7 +7914,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="273" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>260</v>
       </c>
@@ -7921,7 +7922,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="274" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>265</v>
       </c>
@@ -7929,7 +7930,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="275" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>280</v>
       </c>
@@ -7937,7 +7938,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="276" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>282</v>
       </c>
@@ -7945,7 +7946,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="277" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>284</v>
       </c>
@@ -7953,7 +7954,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="278" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>286</v>
       </c>
@@ -7961,7 +7962,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="279" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>288</v>
       </c>
@@ -7969,7 +7970,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="280" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>290</v>
       </c>
@@ -7977,7 +7978,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="281" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>292</v>
       </c>
@@ -7985,7 +7986,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="282" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>296</v>
       </c>
@@ -7993,7 +7994,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="283" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>309</v>
       </c>
@@ -8001,7 +8002,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="284" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>313</v>
       </c>
@@ -8009,7 +8010,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="285" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>315</v>
       </c>
@@ -8017,7 +8018,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="286" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>317</v>
       </c>
@@ -8025,7 +8026,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="287" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>327</v>
       </c>
@@ -8033,7 +8034,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="288" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>335</v>
       </c>
@@ -8041,7 +8042,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="289" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>337</v>
       </c>
@@ -8049,7 +8050,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="290" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>339</v>
       </c>
@@ -8057,7 +8058,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="291" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>341</v>
       </c>
@@ -8065,7 +8066,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="292" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>343</v>
       </c>
@@ -8073,7 +8074,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="293" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>349</v>
       </c>
@@ -8081,7 +8082,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="294" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>351</v>
       </c>
@@ -8089,7 +8090,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="295" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>353</v>
       </c>
@@ -8097,7 +8098,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="296" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>355</v>
       </c>
@@ -8105,7 +8106,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="297" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>357</v>
       </c>
@@ -8113,7 +8114,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="298" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>363</v>
       </c>
@@ -8121,7 +8122,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="299" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>365</v>
       </c>
@@ -8129,7 +8130,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="300" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>367</v>
       </c>
@@ -8137,7 +8138,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="301" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>369</v>
       </c>
@@ -8145,7 +8146,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="302" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>371</v>
       </c>
@@ -8153,7 +8154,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="303" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>374</v>
       </c>
@@ -8161,7 +8162,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="304" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>376</v>
       </c>
@@ -8169,7 +8170,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>378</v>
       </c>
@@ -8177,7 +8178,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>380</v>
       </c>
@@ -8185,7 +8186,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>382</v>
       </c>
@@ -8193,7 +8194,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>386</v>
       </c>
@@ -8201,7 +8202,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>388</v>
       </c>
@@ -8209,7 +8210,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="310" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>390</v>
       </c>
@@ -8217,7 +8218,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="311" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A311" s="2" t="s">
         <v>601</v>
       </c>
@@ -8240,7 +8241,7 @@
         <v>64.705882352941103</v>
       </c>
     </row>
-    <row r="312" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>400</v>
       </c>
@@ -8248,7 +8249,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="313" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>417</v>
       </c>
@@ -8256,7 +8257,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="314" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>420</v>
       </c>
@@ -8264,7 +8265,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="315" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>422</v>
       </c>
@@ -8272,7 +8273,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="316" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>424</v>
       </c>
@@ -8280,7 +8281,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="317" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>426</v>
       </c>
@@ -8288,7 +8289,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="318" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>428</v>
       </c>
@@ -8296,7 +8297,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="319" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>430</v>
       </c>
@@ -8304,7 +8305,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="320" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>432</v>
       </c>
@@ -8312,7 +8313,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="321" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>434</v>
       </c>
@@ -8320,7 +8321,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="322" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>436</v>
       </c>
@@ -8328,7 +8329,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="323" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
         <v>438</v>
       </c>
@@ -8336,7 +8337,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="324" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
         <v>440</v>
       </c>
@@ -8344,7 +8345,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="325" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
         <v>444</v>
       </c>
@@ -8352,7 +8353,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="326" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
         <v>446</v>
       </c>
@@ -8360,7 +8361,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="327" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
         <v>472</v>
       </c>
@@ -8368,7 +8369,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="328" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
         <v>481</v>
       </c>
@@ -8376,7 +8377,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="329" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
         <v>483</v>
       </c>
@@ -8384,7 +8385,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="330" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
         <v>485</v>
       </c>
@@ -8392,7 +8393,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="331" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
         <v>487</v>
       </c>
@@ -8400,7 +8401,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="332" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
         <v>491</v>
       </c>
@@ -8408,7 +8409,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="333" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
         <v>493</v>
       </c>
@@ -8416,7 +8417,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="334" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
         <v>496</v>
       </c>
@@ -8424,7 +8425,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="335" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
         <v>500</v>
       </c>
@@ -8432,7 +8433,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="336" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
         <v>505</v>
       </c>
@@ -8440,7 +8441,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="337" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
         <v>507</v>
       </c>
@@ -8448,7 +8449,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="338" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
         <v>509</v>
       </c>
@@ -8456,7 +8457,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="339" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
         <v>511</v>
       </c>
@@ -8464,7 +8465,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="340" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
         <v>513</v>
       </c>
@@ -8472,7 +8473,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="341" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
         <v>515</v>
       </c>
@@ -8480,7 +8481,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="342" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
         <v>518</v>
       </c>
@@ -8488,7 +8489,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="343" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
         <v>529</v>
       </c>
@@ -8496,7 +8497,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="344" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
         <v>531</v>
       </c>
@@ -8504,7 +8505,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="345" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
         <v>533</v>
       </c>
@@ -8512,7 +8513,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="346" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
         <v>543</v>
       </c>
@@ -8520,7 +8521,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="347" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
         <v>545</v>
       </c>
@@ -8528,7 +8529,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="348" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
         <v>550</v>
       </c>
@@ -8536,7 +8537,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="349" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
         <v>555</v>
       </c>
@@ -8544,7 +8545,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="350" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
         <v>560</v>
       </c>
@@ -8552,7 +8553,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="351" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
         <v>564</v>
       </c>
@@ -8560,7 +8561,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="352" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
         <v>568</v>
       </c>
@@ -8568,7 +8569,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
         <v>570</v>
       </c>
@@ -8576,7 +8577,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
         <v>572</v>
       </c>
@@ -8584,7 +8585,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
         <v>596</v>
       </c>
@@ -8592,7 +8593,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
         <v>604</v>
       </c>
@@ -8600,7 +8601,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
         <v>609</v>
       </c>
@@ -8608,7 +8609,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
         <v>611</v>
       </c>
@@ -8616,7 +8617,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
         <v>613</v>
       </c>
@@ -8624,7 +8625,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
         <v>615</v>
       </c>
@@ -8632,7 +8633,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
         <v>617</v>
       </c>
@@ -8640,7 +8641,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
         <v>627</v>
       </c>
@@ -8648,7 +8649,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
         <v>629</v>
       </c>
@@ -8656,7 +8657,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
         <v>631</v>
       </c>
@@ -8664,7 +8665,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B365">
         <v>10195</v>
       </c>
@@ -8672,7 +8673,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B366">
         <v>10419</v>
       </c>
@@ -8680,7 +8681,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B367">
         <v>10533</v>
       </c>
@@ -8688,7 +8689,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B368">
         <v>10620</v>
       </c>
@@ -8696,7 +8697,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="369" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="369" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B369">
         <v>10626</v>
       </c>
@@ -8704,7 +8705,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="370" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="370" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B370">
         <v>10658</v>
       </c>
@@ -8712,7 +8713,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="371" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="371" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B371" s="4">
         <v>10681</v>
       </c>
@@ -8720,7 +8721,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="372" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="372" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B372">
         <v>10783</v>
       </c>
@@ -8728,7 +8729,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="373" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="373" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B373" s="4">
         <v>10835</v>
       </c>
@@ -8736,7 +8737,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="374" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="374" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B374">
         <v>10838</v>
       </c>
@@ -8744,7 +8745,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="375" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="375" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B375">
         <v>10863</v>
       </c>
@@ -8752,7 +8753,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="376" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="376" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B376" s="4">
         <v>10890</v>
       </c>
@@ -8760,7 +8761,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="377" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="377" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B377">
         <v>10900</v>
       </c>
@@ -8768,7 +8769,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="378" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="378" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B378" s="4">
         <v>10904</v>
       </c>
@@ -8776,7 +8777,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="379" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="379" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B379">
         <v>10909</v>
       </c>
@@ -8784,7 +8785,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="380" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="380" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B380">
         <v>10919</v>
       </c>
@@ -8792,7 +8793,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="381" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="381" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B381">
         <v>10920</v>
       </c>
@@ -8800,7 +8801,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="382" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="382" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B382" s="4">
         <v>10930</v>
       </c>
@@ -8808,7 +8809,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="383" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="383" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B383" s="4">
         <v>11382</v>
       </c>
@@ -8816,7 +8817,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="384" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="384" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B384">
         <v>11389</v>
       </c>
@@ -8824,7 +8825,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="385" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="385" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B385">
         <v>11513</v>
       </c>
@@ -8832,7 +8833,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="386" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="386" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B386">
         <v>11766</v>
       </c>
@@ -8840,7 +8841,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="387" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="387" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B387">
         <v>11767</v>
       </c>
@@ -8848,7 +8849,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="388" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="388" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B388" s="4">
         <v>11804</v>
       </c>
@@ -8856,7 +8857,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="389" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="389" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B389">
         <v>11827</v>
       </c>
@@ -8864,7 +8865,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="390" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="390" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B390">
         <v>11876</v>
       </c>
@@ -8872,7 +8873,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="391" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="391" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B391">
         <v>11981</v>
       </c>
@@ -8880,7 +8881,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="392" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="392" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B392">
         <v>12184</v>
       </c>
@@ -8888,7 +8889,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="393" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="393" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B393" s="4">
         <v>12404</v>
       </c>
@@ -8896,7 +8897,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="394" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="394" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B394">
         <v>12466</v>
       </c>
@@ -8904,7 +8905,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="395" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="395" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B395">
         <v>12660</v>
       </c>
@@ -8912,7 +8913,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="396" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="396" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B396">
         <v>12678</v>
       </c>
@@ -8920,7 +8921,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="397" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="397" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B397">
         <v>12815</v>
       </c>
@@ -8928,7 +8929,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="398" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="398" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B398">
         <v>12841</v>
       </c>
@@ -8936,7 +8937,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="399" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="399" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B399">
         <v>10306</v>
       </c>
@@ -8944,7 +8945,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="400" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="400" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B400">
         <v>10647</v>
       </c>
@@ -8952,7 +8953,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="401" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="401" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B401">
         <v>11046</v>
       </c>
@@ -8960,7 +8961,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="402" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="402" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B402">
         <v>11103</v>
       </c>
@@ -8968,7 +8969,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="403" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="403" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B403">
         <v>11750</v>
       </c>
@@ -8976,7 +8977,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="404" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="404" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B404">
         <v>12555</v>
       </c>
@@ -8985,27 +8986,36 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G404" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:G404" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="Thompson (T-1 and T-3)"/>
+      </filters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:G167">
+      <sortCondition ref="A1:A404"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A9FB282-8562-48BC-8F32-496757DDCE64}">
-  <dimension ref="A1:C263"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C259"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.08984375" customWidth="1"/>
-    <col min="3" max="3" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="63.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" customWidth="1"/>
+    <col min="3" max="3" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="63.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>644</v>
       </c>
@@ -9013,7 +9023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>10011</v>
       </c>
@@ -9021,7 +9031,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>10012</v>
       </c>
@@ -9029,7 +9039,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>10013</v>
       </c>
@@ -9037,7 +9047,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>10014</v>
       </c>
@@ -9045,7 +9055,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>10052</v>
       </c>
@@ -9053,7 +9063,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>10076</v>
       </c>
@@ -9061,7 +9071,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>10091</v>
       </c>
@@ -9069,7 +9079,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>10101</v>
       </c>
@@ -9077,7 +9087,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>10103</v>
       </c>
@@ -9085,7 +9095,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10119</v>
       </c>
@@ -9093,7 +9103,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="12" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>10128</v>
       </c>
@@ -9101,7 +9111,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>10150</v>
       </c>
@@ -9109,7 +9119,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10188</v>
       </c>
@@ -9117,7 +9127,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>10240</v>
       </c>
@@ -9125,7 +9135,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>10275</v>
       </c>
@@ -9133,7 +9143,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>10276</v>
       </c>
@@ -9141,7 +9151,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>10289</v>
       </c>
@@ -9149,7 +9159,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>10295</v>
       </c>
@@ -9157,7 +9167,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>10296</v>
       </c>
@@ -9165,7 +9175,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>10299</v>
       </c>
@@ -9173,7 +9183,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>10300</v>
       </c>
@@ -9181,7 +9191,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>10307</v>
       </c>
@@ -9189,7 +9199,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>10350</v>
       </c>
@@ -9197,7 +9207,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>10369</v>
       </c>
@@ -9205,7 +9215,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>10381</v>
       </c>
@@ -9213,7 +9223,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>10385</v>
       </c>
@@ -9221,7 +9231,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>10398</v>
       </c>
@@ -9229,7 +9239,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>10420</v>
       </c>
@@ -9237,7 +9247,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>10468</v>
       </c>
@@ -9245,7 +9255,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>10569</v>
       </c>
@@ -9253,7 +9263,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>10570</v>
       </c>
@@ -9261,7 +9271,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>10578</v>
       </c>
@@ -9269,7 +9279,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>10579</v>
       </c>
@@ -9277,7 +9287,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>10580</v>
       </c>
@@ -9285,7 +9295,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>10587</v>
       </c>
@@ -9293,7 +9303,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>10589</v>
       </c>
@@ -9301,7 +9311,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>10613</v>
       </c>
@@ -9309,7 +9319,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>10614</v>
       </c>
@@ -9317,7 +9327,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>10617</v>
       </c>
@@ -9325,7 +9335,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>10657</v>
       </c>
@@ -9333,7 +9343,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>10669</v>
       </c>
@@ -9341,7 +9351,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>10678</v>
       </c>
@@ -9349,7 +9359,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>10679</v>
       </c>
@@ -9357,7 +9367,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>10722</v>
       </c>
@@ -9365,7 +9375,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>10738</v>
       </c>
@@ -9373,7 +9383,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>10765</v>
       </c>
@@ -9381,7 +9391,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>10785</v>
       </c>
@@ -9389,7 +9399,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>10791</v>
       </c>
@@ -9397,7 +9407,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>10810</v>
       </c>
@@ -9405,7 +9415,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>10857</v>
       </c>
@@ -9413,7 +9423,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>10873</v>
       </c>
@@ -9421,7 +9431,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>10907</v>
       </c>
@@ -9429,7 +9439,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>10908</v>
       </c>
@@ -9437,7 +9447,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>10911</v>
       </c>
@@ -9445,7 +9455,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>10912</v>
       </c>
@@ -9453,7 +9463,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>10917</v>
       </c>
@@ -9461,7 +9471,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>10922</v>
       </c>
@@ -9469,7 +9479,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>10923</v>
       </c>
@@ -9477,7 +9487,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>10924</v>
       </c>
@@ -9485,7 +9495,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>10926</v>
       </c>
@@ -9493,7 +9503,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>10929</v>
       </c>
@@ -9501,7 +9511,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>10931</v>
       </c>
@@ -9509,7 +9519,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>11368</v>
       </c>
@@ -9517,7 +9527,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>11375</v>
       </c>
@@ -9525,7 +9535,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>11472</v>
       </c>
@@ -9533,7 +9543,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>11496</v>
       </c>
@@ -9541,7 +9551,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>11519</v>
       </c>
@@ -9549,7 +9559,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>11723</v>
       </c>
@@ -9557,7 +9567,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>11730</v>
       </c>
@@ -9565,7 +9575,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>11734</v>
       </c>
@@ -9573,7 +9583,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>11736</v>
       </c>
@@ -9581,7 +9591,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="73" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>11765</v>
       </c>
@@ -9589,7 +9599,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>11770</v>
       </c>
@@ -9597,7 +9607,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>11894</v>
       </c>
@@ -9605,7 +9615,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>11951</v>
       </c>
@@ -9613,7 +9623,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>11989</v>
       </c>
@@ -9621,7 +9631,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>12298</v>
       </c>
@@ -9629,7 +9639,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>12304</v>
       </c>
@@ -9637,7 +9647,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>12459</v>
       </c>
@@ -9645,7 +9655,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>12553</v>
       </c>
@@ -9653,7 +9663,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>10904</v>
       </c>
@@ -9661,7 +9671,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>11804</v>
       </c>
@@ -9669,7 +9679,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>10835</v>
       </c>
@@ -9677,7 +9687,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>11382</v>
       </c>
@@ -9685,7 +9695,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>11794</v>
       </c>
@@ -9693,7 +9703,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>10863</v>
       </c>
@@ -9701,7 +9711,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="5">
         <v>10921</v>
       </c>
@@ -9710,203 +9720,220 @@
       </c>
       <c r="C89" s="5"/>
     </row>
-    <row r="225" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" s="2">
+        <v>10913</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C90" s="2"/>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" s="2">
+        <v>10164</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A221">
+        <v>10419</v>
+      </c>
+    </row>
+    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A222">
+        <v>10533</v>
+      </c>
+    </row>
+    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A223">
+        <v>10620</v>
+      </c>
+    </row>
+    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A224">
+        <v>10626</v>
+      </c>
+    </row>
+    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A225">
-        <v>10419</v>
-      </c>
-    </row>
-    <row r="226" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10658</v>
+      </c>
+    </row>
+    <row r="226" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A226">
-        <v>10533</v>
-      </c>
-    </row>
-    <row r="227" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10681</v>
+      </c>
+    </row>
+    <row r="227" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A227">
-        <v>10620</v>
-      </c>
-    </row>
-    <row r="228" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10783</v>
+      </c>
+    </row>
+    <row r="228" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A228">
-        <v>10626</v>
-      </c>
-    </row>
-    <row r="229" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10835</v>
+      </c>
+    </row>
+    <row r="229" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A229">
-        <v>10658</v>
-      </c>
-    </row>
-    <row r="230" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10838</v>
+      </c>
+    </row>
+    <row r="230" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A230">
-        <v>10681</v>
-      </c>
-    </row>
-    <row r="231" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10863</v>
+      </c>
+    </row>
+    <row r="231" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A231">
-        <v>10783</v>
-      </c>
-    </row>
-    <row r="232" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10890</v>
+      </c>
+    </row>
+    <row r="232" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A232">
-        <v>10835</v>
-      </c>
-    </row>
-    <row r="233" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10900</v>
+      </c>
+    </row>
+    <row r="233" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A233">
-        <v>10838</v>
-      </c>
-    </row>
-    <row r="234" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10904</v>
+      </c>
+    </row>
+    <row r="234" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A234">
-        <v>10863</v>
-      </c>
-    </row>
-    <row r="235" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10909</v>
+      </c>
+    </row>
+    <row r="235" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A235">
-        <v>10890</v>
-      </c>
-    </row>
-    <row r="236" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10919</v>
+      </c>
+    </row>
+    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A236">
-        <v>10900</v>
-      </c>
-    </row>
-    <row r="237" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10920</v>
+      </c>
+    </row>
+    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A237">
-        <v>10904</v>
-      </c>
-    </row>
-    <row r="238" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10930</v>
+      </c>
+    </row>
+    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A238">
-        <v>10909</v>
-      </c>
-    </row>
-    <row r="239" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11382</v>
+      </c>
+    </row>
+    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A239">
-        <v>10919</v>
-      </c>
-    </row>
-    <row r="240" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11389</v>
+      </c>
+    </row>
+    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A240">
-        <v>10920</v>
-      </c>
-    </row>
-    <row r="241" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11513</v>
+      </c>
+    </row>
+    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A241">
-        <v>10930</v>
-      </c>
-    </row>
-    <row r="242" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11766</v>
+      </c>
+    </row>
+    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A242">
-        <v>11382</v>
-      </c>
-    </row>
-    <row r="243" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11767</v>
+      </c>
+    </row>
+    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A243">
-        <v>11389</v>
-      </c>
-    </row>
-    <row r="244" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11804</v>
+      </c>
+    </row>
+    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A244">
-        <v>11513</v>
-      </c>
-    </row>
-    <row r="245" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11827</v>
+      </c>
+    </row>
+    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A245">
-        <v>11766</v>
-      </c>
-    </row>
-    <row r="246" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11876</v>
+      </c>
+    </row>
+    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A246">
-        <v>11767</v>
-      </c>
-    </row>
-    <row r="247" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11981</v>
+      </c>
+    </row>
+    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A247">
-        <v>11804</v>
-      </c>
-    </row>
-    <row r="248" spans="1:1" x14ac:dyDescent="0.35">
+        <v>12184</v>
+      </c>
+    </row>
+    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A248">
-        <v>11827</v>
-      </c>
-    </row>
-    <row r="249" spans="1:1" x14ac:dyDescent="0.35">
+        <v>12404</v>
+      </c>
+    </row>
+    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A249">
-        <v>11876</v>
-      </c>
-    </row>
-    <row r="250" spans="1:1" x14ac:dyDescent="0.35">
+        <v>12466</v>
+      </c>
+    </row>
+    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A250">
-        <v>11981</v>
-      </c>
-    </row>
-    <row r="251" spans="1:1" x14ac:dyDescent="0.35">
+        <v>12660</v>
+      </c>
+    </row>
+    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A251">
-        <v>12184</v>
-      </c>
-    </row>
-    <row r="252" spans="1:1" x14ac:dyDescent="0.35">
+        <v>12678</v>
+      </c>
+    </row>
+    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A252">
-        <v>12404</v>
-      </c>
-    </row>
-    <row r="253" spans="1:1" x14ac:dyDescent="0.35">
+        <v>12815</v>
+      </c>
+    </row>
+    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A253">
-        <v>12466</v>
-      </c>
-    </row>
-    <row r="254" spans="1:1" x14ac:dyDescent="0.35">
+        <v>12841</v>
+      </c>
+    </row>
+    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A254">
-        <v>12660</v>
-      </c>
-    </row>
-    <row r="255" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10306</v>
+      </c>
+    </row>
+    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A255">
-        <v>12678</v>
-      </c>
-    </row>
-    <row r="256" spans="1:1" x14ac:dyDescent="0.35">
+        <v>10647</v>
+      </c>
+    </row>
+    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A256">
-        <v>12815</v>
-      </c>
-    </row>
-    <row r="257" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11046</v>
+      </c>
+    </row>
+    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A257">
-        <v>12841</v>
-      </c>
-    </row>
-    <row r="258" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11103</v>
+      </c>
+    </row>
+    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A258">
-        <v>10306</v>
-      </c>
-    </row>
-    <row r="259" spans="1:1" x14ac:dyDescent="0.35">
+        <v>11750</v>
+      </c>
+    </row>
+    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A259">
-        <v>10647</v>
-      </c>
-    </row>
-    <row r="260" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A260">
-        <v>11046</v>
-      </c>
-    </row>
-    <row r="261" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A261">
-        <v>11103</v>
-      </c>
-    </row>
-    <row r="262" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A262">
-        <v>11750</v>
-      </c>
-    </row>
-    <row r="263" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A263">
         <v>12555</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B89" xr:uid="{9A9FB282-8562-48BC-8F32-496757DDCE64}"/>
+  <autoFilter ref="A1:B91" xr:uid="{9A9FB282-8562-48BC-8F32-496757DDCE64}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added carbon stock ecosystems table - small format change
</commit_message>
<xml_diff>
--- a/data/Mappings/mapping_ghg.xlsx
+++ b/data/Mappings/mapping_ghg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca-my.sharepoint.com/personal/marin_pellan_polymtl_ca/Documents/POST_DOC/CODE/metallican_db/data/Mappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="321" documentId="11_F25DC773A252ABDACC104887411C794C5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B593DDF9-079C-45D5-A9CC-91D11B21CCBA}"/>
+  <xr:revisionPtr revIDLastSave="322" documentId="11_F25DC773A252ABDACC104887411C794C5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E996556-0C19-46B0-AB2E-2666A78BAF16}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LT" sheetId="1" r:id="rId1"/>
@@ -2179,10 +2179,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2448,7 +2444,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G404"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2484,7 +2479,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>191</v>
       </c>
@@ -2507,7 +2502,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>359</v>
       </c>
@@ -2530,7 +2525,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>576</v>
       </c>
@@ -2553,7 +2548,7 @@
         <v>20.689655172413701</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>591</v>
       </c>
@@ -2576,7 +2571,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -2599,7 +2594,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>361</v>
       </c>
@@ -2622,7 +2617,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>463</v>
       </c>
@@ -2645,7 +2640,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>85</v>
       </c>
@@ -2668,7 +2663,7 @@
         <v>54.545454545454497</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>442</v>
       </c>
@@ -2691,7 +2686,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>395</v>
       </c>
@@ -2704,7 +2699,7 @@
       <c r="F11"/>
       <c r="G11"/>
     </row>
-    <row r="12" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>324</v>
       </c>
@@ -2727,7 +2722,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>255</v>
       </c>
@@ -2750,7 +2745,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>453</v>
       </c>
@@ -2773,7 +2768,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>539</v>
       </c>
@@ -2796,7 +2791,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>580</v>
       </c>
@@ -2819,7 +2814,7 @@
         <v>16.6666666666666</v>
       </c>
     </row>
-    <row r="17" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>467</v>
       </c>
@@ -2842,7 +2837,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>48</v>
       </c>
@@ -2865,7 +2860,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>298</v>
       </c>
@@ -2888,7 +2883,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>477</v>
       </c>
@@ -2911,7 +2906,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>465</v>
       </c>
@@ -2934,7 +2929,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="22" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>202</v>
       </c>
@@ -2957,7 +2952,7 @@
         <v>58.823529411764703</v>
       </c>
     </row>
-    <row r="23" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>547</v>
       </c>
@@ -2980,7 +2975,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="24" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>552</v>
       </c>
@@ -3003,7 +2998,7 @@
         <v>37.5</v>
       </c>
     </row>
-    <row r="25" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>582</v>
       </c>
@@ -3026,7 +3021,7 @@
         <v>15.6862745098039</v>
       </c>
     </row>
-    <row r="26" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>43</v>
       </c>
@@ -3049,7 +3044,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>502</v>
       </c>
@@ -3072,7 +3067,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="28" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>586</v>
       </c>
@@ -3095,7 +3090,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="29" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>85</v>
       </c>
@@ -3118,7 +3113,7 @@
         <v>56.521739130434703</v>
       </c>
     </row>
-    <row r="30" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>250</v>
       </c>
@@ -3141,7 +3136,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="31" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>63</v>
       </c>
@@ -3164,7 +3159,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>112</v>
       </c>
@@ -3187,7 +3182,7 @@
         <v>55.172413793103402</v>
       </c>
     </row>
-    <row r="33" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>59</v>
       </c>
@@ -3210,7 +3205,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>15</v>
       </c>
@@ -3233,7 +3228,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>45</v>
       </c>
@@ -3256,7 +3251,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>245</v>
       </c>
@@ -3279,7 +3274,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="37" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>562</v>
       </c>
@@ -3302,7 +3297,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="38" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>412</v>
       </c>
@@ -3325,7 +3320,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="39" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>448</v>
       </c>
@@ -3348,7 +3343,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>402</v>
       </c>
@@ -3371,7 +3366,7 @@
         <v>23.529411764705799</v>
       </c>
     </row>
-    <row r="41" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>584</v>
       </c>
@@ -3394,7 +3389,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="42" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>465</v>
       </c>
@@ -3417,7 +3412,7 @@
         <v>18.518518518518501</v>
       </c>
     </row>
-    <row r="43" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>589</v>
       </c>
@@ -3440,7 +3435,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="44" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>479</v>
       </c>
@@ -3463,7 +3458,7 @@
         <v>34.567901234567898</v>
       </c>
     </row>
-    <row r="45" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>474</v>
       </c>
@@ -3486,7 +3481,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>74</v>
       </c>
@@ -3509,7 +3504,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="47" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>252</v>
       </c>
@@ -3532,7 +3527,7 @@
         <v>15.0537634408602</v>
       </c>
     </row>
-    <row r="48" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>87</v>
       </c>
@@ -3555,7 +3550,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="49" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>121</v>
       </c>
@@ -3578,7 +3573,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="50" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>199</v>
       </c>
@@ -3601,7 +3596,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="51" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>456</v>
       </c>
@@ -3624,7 +3619,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>470</v>
       </c>
@@ -3647,7 +3642,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>248</v>
       </c>
@@ -3670,7 +3665,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="54" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>450</v>
       </c>
@@ -3693,7 +3688,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>460</v>
       </c>
@@ -3716,7 +3711,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="56" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>589</v>
       </c>
@@ -3739,7 +3734,7 @@
         <v>7.1428571428571299</v>
       </c>
     </row>
-    <row r="57" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>241</v>
       </c>
@@ -3762,7 +3757,7 @@
         <v>57.142857142857103</v>
       </c>
     </row>
-    <row r="58" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>456</v>
       </c>
@@ -3785,7 +3780,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="59" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>456</v>
       </c>
@@ -3808,7 +3803,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>262</v>
       </c>
@@ -3831,7 +3826,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="61" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>598</v>
       </c>
@@ -3854,7 +3849,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="62" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>51</v>
       </c>
@@ -3877,7 +3872,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="63" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>238</v>
       </c>
@@ -3900,7 +3895,7 @@
         <v>26.6666666666666</v>
       </c>
     </row>
-    <row r="64" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>321</v>
       </c>
@@ -3923,7 +3918,7 @@
         <v>33.3333333333333</v>
       </c>
     </row>
-    <row r="65" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>28</v>
       </c>
@@ -3946,7 +3941,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="66" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>19</v>
       </c>
@@ -3969,7 +3964,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="67" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>522</v>
       </c>
@@ -3992,7 +3987,7 @@
         <v>20.8333333333333</v>
       </c>
     </row>
-    <row r="68" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>409</v>
       </c>
@@ -4015,7 +4010,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>537</v>
       </c>
@@ -4038,7 +4033,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>31</v>
       </c>
@@ -4061,7 +4056,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="71" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>63</v>
       </c>
@@ -4084,7 +4079,7 @@
         <v>66.6666666666666</v>
       </c>
     </row>
-    <row r="72" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>77</v>
       </c>
@@ -4107,7 +4102,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="73" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>465</v>
       </c>
@@ -4130,7 +4125,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>170</v>
       </c>
@@ -4153,7 +4148,7 @@
         <v>33.3333333333333</v>
       </c>
     </row>
-    <row r="75" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>59</v>
       </c>
@@ -4176,7 +4171,7 @@
         <v>23.076923076922998</v>
       </c>
     </row>
-    <row r="76" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>127</v>
       </c>
@@ -4199,7 +4194,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="77" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>566</v>
       </c>
@@ -4222,7 +4217,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="78" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>524</v>
       </c>
@@ -4245,7 +4240,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>90</v>
       </c>
@@ -4268,7 +4263,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>541</v>
       </c>
@@ -4291,7 +4286,7 @@
         <v>55.172413793103402</v>
       </c>
     </row>
-    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>257</v>
       </c>
@@ -4314,7 +4309,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="82" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>196</v>
       </c>
@@ -4337,7 +4332,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>51</v>
       </c>
@@ -4360,7 +4355,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>522</v>
       </c>
@@ -4383,7 +4378,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>522</v>
       </c>
@@ -4406,7 +4401,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>51</v>
       </c>
@@ -4429,7 +4424,7 @@
         <v>7.8431372549019596</v>
       </c>
     </row>
-    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>90</v>
       </c>
@@ -4452,7 +4447,7 @@
         <v>29.090909090909001</v>
       </c>
     </row>
-    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>202</v>
       </c>
@@ -4475,7 +4470,7 @@
         <v>48.8888888888888</v>
       </c>
     </row>
-    <row r="89" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>495</v>
       </c>
@@ -4498,7 +4493,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>527</v>
       </c>
@@ -4521,7 +4516,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>319</v>
       </c>
@@ -4544,7 +4539,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>174</v>
       </c>
@@ -4567,7 +4562,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>333</v>
       </c>
@@ -4590,7 +4585,7 @@
         <v>21.052631578947299</v>
       </c>
     </row>
-    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>319</v>
       </c>
@@ -4613,7 +4608,7 @@
         <v>37.037037037037003</v>
       </c>
     </row>
-    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>90</v>
       </c>
@@ -4636,7 +4631,7 @@
         <v>76.470588235294102</v>
       </c>
     </row>
-    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>392</v>
       </c>
@@ -4659,7 +4654,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="97" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>606</v>
       </c>
@@ -4682,7 +4677,7 @@
         <v>51.428571428571402</v>
       </c>
     </row>
-    <row r="98" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>522</v>
       </c>
@@ -4705,7 +4700,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>90</v>
       </c>
@@ -4728,7 +4723,7 @@
         <v>20.689655172413701</v>
       </c>
     </row>
-    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>267</v>
       </c>
@@ -4751,7 +4746,7 @@
         <v>54.545454545454497</v>
       </c>
     </row>
-    <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>130</v>
       </c>
@@ -4774,7 +4769,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>90</v>
       </c>
@@ -4797,7 +4792,7 @@
         <v>23.8095238095238</v>
       </c>
     </row>
-    <row r="103" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>519</v>
       </c>
@@ -4820,7 +4815,7 @@
         <v>27.7777777777777</v>
       </c>
     </row>
-    <row r="104" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>397</v>
       </c>
@@ -4843,7 +4838,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="105" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>156</v>
       </c>
@@ -4866,7 +4861,7 @@
         <v>66.6666666666666</v>
       </c>
     </row>
-    <row r="106" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>623</v>
       </c>
@@ -4889,7 +4884,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="107" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>81</v>
       </c>
@@ -4912,7 +4907,7 @@
         <v>59.090909090909001</v>
       </c>
     </row>
-    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>302</v>
       </c>
@@ -4935,7 +4930,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>81</v>
       </c>
@@ -4958,7 +4953,7 @@
         <v>52.173913043478201</v>
       </c>
     </row>
-    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>557</v>
       </c>
@@ -4981,7 +4976,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>191</v>
       </c>
@@ -5004,7 +4999,7 @@
         <v>21.428571428571399</v>
       </c>
     </row>
-    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>465</v>
       </c>
@@ -5027,7 +5022,7 @@
         <v>19.354838709677399</v>
       </c>
     </row>
-    <row r="113" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>406</v>
       </c>
@@ -5050,7 +5045,7 @@
         <v>12.1212121212121</v>
       </c>
     </row>
-    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>191</v>
       </c>
@@ -5073,7 +5068,7 @@
         <v>19.672131147540899</v>
       </c>
     </row>
-    <row r="115" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="4" t="s">
         <v>24</v>
       </c>
@@ -5096,7 +5091,7 @@
         <v>52.173913043478201</v>
       </c>
     </row>
-    <row r="116" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>414</v>
       </c>
@@ -5119,7 +5114,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="117" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>300</v>
       </c>
@@ -5142,7 +5137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:7" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>522</v>
       </c>
@@ -5165,7 +5160,7 @@
         <v>72.727272727272705</v>
       </c>
     </row>
-    <row r="119" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>456</v>
       </c>
@@ -5188,7 +5183,7 @@
         <v>14.285714285714199</v>
       </c>
     </row>
-    <row r="120" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>191</v>
       </c>
@@ -5211,7 +5206,7 @@
         <v>25.806451612903199</v>
       </c>
     </row>
-    <row r="121" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>489</v>
       </c>
@@ -5234,7 +5229,7 @@
         <v>30.769230769230699</v>
       </c>
     </row>
-    <row r="122" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>576</v>
       </c>
@@ -5257,7 +5252,7 @@
         <v>34.285714285714199</v>
       </c>
     </row>
-    <row r="123" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>71</v>
       </c>
@@ -5280,7 +5275,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="124" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>51</v>
       </c>
@@ -5303,7 +5298,7 @@
         <v>14.285714285714199</v>
       </c>
     </row>
-    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>305</v>
       </c>
@@ -5326,7 +5321,7 @@
         <v>57.142857142857103</v>
       </c>
     </row>
-    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>621</v>
       </c>
@@ -5349,7 +5344,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>148</v>
       </c>
@@ -5357,7 +5352,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>541</v>
       </c>
@@ -5380,7 +5375,7 @@
         <v>40.909090909090899</v>
       </c>
     </row>
-    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>100</v>
       </c>
@@ -5403,7 +5398,7 @@
         <v>6.6666666666666696</v>
       </c>
     </row>
-    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>406</v>
       </c>
@@ -5426,7 +5421,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>402</v>
       </c>
@@ -5449,7 +5444,7 @@
         <v>41.379310344827502</v>
       </c>
     </row>
-    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>194</v>
       </c>
@@ -5472,7 +5467,7 @@
         <v>31.25</v>
       </c>
     </row>
-    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>384</v>
       </c>
@@ -5495,7 +5490,7 @@
         <v>23.076923076922998</v>
       </c>
     </row>
-    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>539</v>
       </c>
@@ -5518,7 +5513,7 @@
         <v>10.5263157894736</v>
       </c>
     </row>
-    <row r="135" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>270</v>
       </c>
@@ -5541,7 +5536,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>412</v>
       </c>
@@ -5564,7 +5559,7 @@
         <v>17.647058823529399</v>
       </c>
     </row>
-    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>136</v>
       </c>
@@ -5572,7 +5567,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>194</v>
       </c>
@@ -5595,7 +5590,7 @@
         <v>46.511627906976699</v>
       </c>
     </row>
-    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>384</v>
       </c>
@@ -5618,7 +5613,7 @@
         <v>31.746031746031701</v>
       </c>
     </row>
-    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>448</v>
       </c>
@@ -5641,7 +5636,7 @@
         <v>30.303030303030202</v>
       </c>
     </row>
-    <row r="141" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>24</v>
       </c>
@@ -5664,7 +5659,7 @@
         <v>42.857142857142797</v>
       </c>
     </row>
-    <row r="142" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>24</v>
       </c>
@@ -5687,7 +5682,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>170</v>
       </c>
@@ -5710,7 +5705,7 @@
         <v>20.8333333333333</v>
       </c>
     </row>
-    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>100</v>
       </c>
@@ -5733,7 +5728,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>255</v>
       </c>
@@ -5756,7 +5751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>319</v>
       </c>
@@ -5779,7 +5774,7 @@
         <v>26.6666666666666</v>
       </c>
     </row>
-    <row r="147" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>307</v>
       </c>
@@ -5802,7 +5797,7 @@
         <v>23.529411764705799</v>
       </c>
     </row>
-    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>100</v>
       </c>
@@ -5825,7 +5820,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>156</v>
       </c>
@@ -5848,7 +5843,7 @@
         <v>20.689655172413701</v>
       </c>
     </row>
-    <row r="150" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>498</v>
       </c>
@@ -5871,7 +5866,7 @@
         <v>9.0909090909090899</v>
       </c>
     </row>
-    <row r="151" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>272</v>
       </c>
@@ -5894,7 +5889,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>347</v>
       </c>
@@ -5917,7 +5912,7 @@
         <v>25.6410256410256</v>
       </c>
     </row>
-    <row r="153" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>329</v>
       </c>
@@ -5940,7 +5935,7 @@
         <v>66.6666666666666</v>
       </c>
     </row>
-    <row r="154" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>96</v>
       </c>
@@ -5963,7 +5958,7 @@
         <v>27.272727272727199</v>
       </c>
     </row>
-    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>187</v>
       </c>
@@ -5986,7 +5981,7 @@
         <v>9.0909090909090899</v>
       </c>
     </row>
-    <row r="156" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>587</v>
       </c>
@@ -6009,7 +6004,7 @@
         <v>23.728813559321999</v>
       </c>
     </row>
-    <row r="157" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>591</v>
       </c>
@@ -6032,7 +6027,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="158" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>234</v>
       </c>
@@ -6055,7 +6050,7 @@
         <v>27.118644067796598</v>
       </c>
     </row>
-    <row r="159" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>40</v>
       </c>
@@ -6078,7 +6073,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="160" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>359</v>
       </c>
@@ -6101,7 +6096,7 @@
         <v>26.229508196721302</v>
       </c>
     </row>
-    <row r="161" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>412</v>
       </c>
@@ -6124,7 +6119,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="162" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>361</v>
       </c>
@@ -6147,7 +6142,7 @@
         <v>11.764705882352899</v>
       </c>
     </row>
-    <row r="163" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>51</v>
       </c>
@@ -6170,7 +6165,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="164" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>448</v>
       </c>
@@ -6193,7 +6188,7 @@
         <v>26.6666666666666</v>
       </c>
     </row>
-    <row r="165" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>456</v>
       </c>
@@ -6216,7 +6211,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="166" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="5" t="s">
         <v>311</v>
       </c>
@@ -6239,7 +6234,7 @@
         <v>57.142857142857103</v>
       </c>
     </row>
-    <row r="167" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
         <v>133</v>
       </c>
@@ -6262,7 +6257,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="168" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>465</v>
       </c>
@@ -6285,7 +6280,7 @@
         <v>26.086956521739101</v>
       </c>
     </row>
-    <row r="169" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>359</v>
       </c>
@@ -6308,7 +6303,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="170" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>77</v>
       </c>
@@ -6331,7 +6326,7 @@
         <v>14.285714285714199</v>
       </c>
     </row>
-    <row r="171" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>361</v>
       </c>
@@ -6354,7 +6349,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="172" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>359</v>
       </c>
@@ -6377,7 +6372,7 @@
         <v>32.258064516128997</v>
       </c>
     </row>
-    <row r="173" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>361</v>
       </c>
@@ -6400,7 +6395,7 @@
         <v>19.047619047619001</v>
       </c>
     </row>
-    <row r="174" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>625</v>
       </c>
@@ -6423,7 +6418,7 @@
         <v>17.7777777777777</v>
       </c>
     </row>
-    <row r="175" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>463</v>
       </c>
@@ -6446,7 +6441,7 @@
         <v>18.75</v>
       </c>
     </row>
-    <row r="176" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>178</v>
       </c>
@@ -6469,7 +6464,7 @@
         <v>18.75</v>
       </c>
     </row>
-    <row r="177" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>241</v>
       </c>
@@ -6492,7 +6487,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="178" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>191</v>
       </c>
@@ -6515,7 +6510,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="179" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>250</v>
       </c>
@@ -6538,7 +6533,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="180" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>591</v>
       </c>
@@ -6561,7 +6556,7 @@
         <v>26.6666666666666</v>
       </c>
     </row>
-    <row r="181" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>576</v>
       </c>
@@ -6584,7 +6579,7 @@
         <v>23.529411764705799</v>
       </c>
     </row>
-    <row r="182" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>359</v>
       </c>
@@ -6607,7 +6602,7 @@
         <v>26.315789473684202</v>
       </c>
     </row>
-    <row r="183" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>191</v>
       </c>
@@ -6630,7 +6625,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="184" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>361</v>
       </c>
@@ -6653,7 +6648,7 @@
         <v>21.428571428571399</v>
       </c>
     </row>
-    <row r="185" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>448</v>
       </c>
@@ -6676,7 +6671,7 @@
         <v>11.4285714285714</v>
       </c>
     </row>
-    <row r="186" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>402</v>
       </c>
@@ -6699,7 +6694,7 @@
         <v>29.629629629629601</v>
       </c>
     </row>
-    <row r="187" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
         <v>619</v>
       </c>
@@ -6722,7 +6717,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="188" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>463</v>
       </c>
@@ -6745,7 +6740,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="189" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>463</v>
       </c>
@@ -6768,7 +6763,7 @@
         <v>27.272727272727199</v>
       </c>
     </row>
-    <row r="190" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
         <v>406</v>
       </c>
@@ -6791,7 +6786,7 @@
         <v>46.6666666666666</v>
       </c>
     </row>
-    <row r="191" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>465</v>
       </c>
@@ -6814,7 +6809,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="192" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>329</v>
       </c>
@@ -6837,7 +6832,7 @@
         <v>19.354838709677399</v>
       </c>
     </row>
-    <row r="193" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>456</v>
       </c>
@@ -6860,7 +6855,7 @@
         <v>18.181818181818102</v>
       </c>
     </row>
-    <row r="194" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>463</v>
       </c>
@@ -6883,7 +6878,7 @@
         <v>21.818181818181799</v>
       </c>
     </row>
-    <row r="195" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>574</v>
       </c>
@@ -6906,7 +6901,7 @@
         <v>26.315789473684202</v>
       </c>
     </row>
-    <row r="196" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>51</v>
       </c>
@@ -6929,7 +6924,7 @@
         <v>18.181818181818102</v>
       </c>
     </row>
-    <row r="197" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>458</v>
       </c>
@@ -6952,7 +6947,7 @@
         <v>29.629629629629601</v>
       </c>
     </row>
-    <row r="198" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>535</v>
       </c>
@@ -6975,7 +6970,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="199" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>621</v>
       </c>
@@ -6998,7 +6993,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="200" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>100</v>
       </c>
@@ -7021,7 +7016,7 @@
         <v>22.2222222222222</v>
       </c>
     </row>
-    <row r="201" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>412</v>
       </c>
@@ -7044,7 +7039,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="202" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>347</v>
       </c>
@@ -7067,7 +7062,7 @@
         <v>24.5614035087719</v>
       </c>
     </row>
-    <row r="203" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>5</v>
       </c>
@@ -7090,7 +7085,7 @@
         <v>27.7777777777777</v>
       </c>
     </row>
-    <row r="204" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>234</v>
       </c>
@@ -7113,7 +7108,7 @@
         <v>16.326530612244799</v>
       </c>
     </row>
-    <row r="205" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>234</v>
       </c>
@@ -7136,7 +7131,7 @@
         <v>4.6511627906976596</v>
       </c>
     </row>
-    <row r="206" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>489</v>
       </c>
@@ -7159,7 +7154,7 @@
         <v>5.8823529411764603</v>
       </c>
     </row>
-    <row r="207" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>406</v>
       </c>
@@ -7182,7 +7177,7 @@
         <v>22.857142857142801</v>
       </c>
     </row>
-    <row r="208" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>234</v>
       </c>
@@ -7205,7 +7200,7 @@
         <v>28.571428571428498</v>
       </c>
     </row>
-    <row r="209" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>347</v>
       </c>
@@ -7228,7 +7223,7 @@
         <v>20.689655172413701</v>
       </c>
     </row>
-    <row r="210" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>48</v>
       </c>
@@ -7251,7 +7246,7 @@
         <v>15.3846153846153</v>
       </c>
     </row>
-    <row r="211" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>276</v>
       </c>
@@ -7274,7 +7269,7 @@
         <v>18.518518518518501</v>
       </c>
     </row>
-    <row r="212" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>347</v>
       </c>
@@ -7297,7 +7292,7 @@
         <v>8.6956521739130395</v>
       </c>
     </row>
-    <row r="213" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>345</v>
       </c>
@@ -7320,7 +7315,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="214" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>458</v>
       </c>
@@ -7343,7 +7338,7 @@
         <v>12.1212121212121</v>
       </c>
     </row>
-    <row r="215" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>294</v>
       </c>
@@ -7366,7 +7361,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="216" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>22</v>
       </c>
@@ -7389,7 +7384,7 @@
         <v>14.285714285714199</v>
       </c>
     </row>
-    <row r="217" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>15</v>
       </c>
@@ -7412,7 +7407,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="218" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>402</v>
       </c>
@@ -7435,7 +7430,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="219" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
         <v>450</v>
       </c>
@@ -7458,7 +7453,7 @@
         <v>73.684210526315795</v>
       </c>
     </row>
-    <row r="220" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>8</v>
       </c>
@@ -7466,7 +7461,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="221" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>10</v>
       </c>
@@ -7474,7 +7469,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="222" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>13</v>
       </c>
@@ -7482,7 +7477,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="223" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
         <v>34</v>
       </c>
@@ -7492,7 +7487,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="224" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>36</v>
       </c>
@@ -7500,7 +7495,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="225" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>38</v>
       </c>
@@ -7508,7 +7503,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="226" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>67</v>
       </c>
@@ -7516,7 +7511,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="227" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>69</v>
       </c>
@@ -7524,7 +7519,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="228" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>98</v>
       </c>
@@ -7532,7 +7527,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="229" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>106</v>
       </c>
@@ -7540,7 +7535,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="230" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>108</v>
       </c>
@@ -7548,7 +7543,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="231" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>110</v>
       </c>
@@ -7556,7 +7551,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="232" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>115</v>
       </c>
@@ -7564,7 +7559,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="233" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>117</v>
       </c>
@@ -7572,7 +7567,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="234" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>119</v>
       </c>
@@ -7580,7 +7575,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="235" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>123</v>
       </c>
@@ -7588,7 +7583,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="236" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>125</v>
       </c>
@@ -7596,7 +7591,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="237" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A237" s="2" t="s">
         <v>278</v>
       </c>
@@ -7619,7 +7614,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="238" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>138</v>
       </c>
@@ -7627,7 +7622,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="239" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>140</v>
       </c>
@@ -7635,7 +7630,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="240" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>142</v>
       </c>
@@ -7643,7 +7638,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="241" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>144</v>
       </c>
@@ -7651,7 +7646,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="242" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>146</v>
       </c>
@@ -7682,7 +7677,7 @@
         <v>59.259259259259203</v>
       </c>
     </row>
-    <row r="244" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>150</v>
       </c>
@@ -7690,7 +7685,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="245" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>152</v>
       </c>
@@ -7698,7 +7693,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="246" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>154</v>
       </c>
@@ -7706,7 +7701,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="247" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>158</v>
       </c>
@@ -7714,7 +7709,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="248" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>160</v>
       </c>
@@ -7722,7 +7717,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="249" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>162</v>
       </c>
@@ -7730,7 +7725,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="250" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>164</v>
       </c>
@@ -7738,7 +7733,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="251" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>166</v>
       </c>
@@ -7746,7 +7741,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="252" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>168</v>
       </c>
@@ -7754,7 +7749,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="253" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>176</v>
       </c>
@@ -7762,7 +7757,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="254" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>181</v>
       </c>
@@ -7770,7 +7765,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="255" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>183</v>
       </c>
@@ -7778,7 +7773,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="256" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>185</v>
       </c>
@@ -7786,7 +7781,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="257" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>189</v>
       </c>
@@ -7794,7 +7789,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="258" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>204</v>
       </c>
@@ -7802,7 +7797,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="259" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>206</v>
       </c>
@@ -7810,7 +7805,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="260" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>208</v>
       </c>
@@ -7818,7 +7813,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="261" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>210</v>
       </c>
@@ -7826,7 +7821,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="262" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>212</v>
       </c>
@@ -7834,7 +7829,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="263" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>214</v>
       </c>
@@ -7842,7 +7837,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="264" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>216</v>
       </c>
@@ -7850,7 +7845,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="265" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>218</v>
       </c>
@@ -7858,7 +7853,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="266" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>220</v>
       </c>
@@ -7866,7 +7861,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="267" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>222</v>
       </c>
@@ -7874,7 +7869,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="268" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>224</v>
       </c>
@@ -7882,7 +7877,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="269" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>226</v>
       </c>
@@ -7890,7 +7885,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="270" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>228</v>
       </c>
@@ -7898,7 +7893,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="271" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>230</v>
       </c>
@@ -7906,7 +7901,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="272" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>232</v>
       </c>
@@ -7914,7 +7909,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="273" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>260</v>
       </c>
@@ -7922,7 +7917,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="274" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>265</v>
       </c>
@@ -7930,7 +7925,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="275" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>280</v>
       </c>
@@ -7938,7 +7933,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="276" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>282</v>
       </c>
@@ -7946,7 +7941,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="277" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>284</v>
       </c>
@@ -7954,7 +7949,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="278" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>286</v>
       </c>
@@ -7962,7 +7957,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="279" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>288</v>
       </c>
@@ -7970,7 +7965,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="280" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>290</v>
       </c>
@@ -7978,7 +7973,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="281" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>292</v>
       </c>
@@ -7986,7 +7981,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="282" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>296</v>
       </c>
@@ -7994,7 +7989,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="283" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>309</v>
       </c>
@@ -8002,7 +7997,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="284" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>313</v>
       </c>
@@ -8010,7 +8005,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="285" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>315</v>
       </c>
@@ -8018,7 +8013,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="286" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>317</v>
       </c>
@@ -8026,7 +8021,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="287" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>327</v>
       </c>
@@ -8034,7 +8029,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="288" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>335</v>
       </c>
@@ -8042,7 +8037,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="289" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>337</v>
       </c>
@@ -8050,7 +8045,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="290" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>339</v>
       </c>
@@ -8058,7 +8053,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="291" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>341</v>
       </c>
@@ -8066,7 +8061,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="292" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>343</v>
       </c>
@@ -8074,7 +8069,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="293" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>349</v>
       </c>
@@ -8082,7 +8077,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="294" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>351</v>
       </c>
@@ -8090,7 +8085,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="295" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>353</v>
       </c>
@@ -8098,7 +8093,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="296" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>355</v>
       </c>
@@ -8106,7 +8101,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="297" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>357</v>
       </c>
@@ -8114,7 +8109,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="298" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>363</v>
       </c>
@@ -8122,7 +8117,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="299" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>365</v>
       </c>
@@ -8130,7 +8125,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="300" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>367</v>
       </c>
@@ -8138,7 +8133,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="301" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>369</v>
       </c>
@@ -8146,7 +8141,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="302" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>371</v>
       </c>
@@ -8154,7 +8149,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="303" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>374</v>
       </c>
@@ -8162,7 +8157,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="304" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>376</v>
       </c>
@@ -8170,7 +8165,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="305" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>378</v>
       </c>
@@ -8178,7 +8173,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="306" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>380</v>
       </c>
@@ -8186,7 +8181,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="307" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>382</v>
       </c>
@@ -8194,7 +8189,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="308" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>386</v>
       </c>
@@ -8202,7 +8197,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="309" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>388</v>
       </c>
@@ -8210,7 +8205,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="310" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>390</v>
       </c>
@@ -8218,7 +8213,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="311" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A311" s="2" t="s">
         <v>601</v>
       </c>
@@ -8241,7 +8236,7 @@
         <v>64.705882352941103</v>
       </c>
     </row>
-    <row r="312" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>400</v>
       </c>
@@ -8249,7 +8244,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="313" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>417</v>
       </c>
@@ -8257,7 +8252,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="314" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>420</v>
       </c>
@@ -8265,7 +8260,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="315" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>422</v>
       </c>
@@ -8273,7 +8268,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="316" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>424</v>
       </c>
@@ -8281,7 +8276,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="317" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>426</v>
       </c>
@@ -8289,7 +8284,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="318" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>428</v>
       </c>
@@ -8297,7 +8292,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="319" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>430</v>
       </c>
@@ -8305,7 +8300,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="320" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>432</v>
       </c>
@@ -8313,7 +8308,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="321" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>434</v>
       </c>
@@ -8321,7 +8316,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="322" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>436</v>
       </c>
@@ -8329,7 +8324,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="323" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
         <v>438</v>
       </c>
@@ -8337,7 +8332,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="324" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
         <v>440</v>
       </c>
@@ -8345,7 +8340,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="325" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
         <v>444</v>
       </c>
@@ -8353,7 +8348,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="326" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
         <v>446</v>
       </c>
@@ -8361,7 +8356,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="327" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
         <v>472</v>
       </c>
@@ -8369,7 +8364,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="328" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
         <v>481</v>
       </c>
@@ -8377,7 +8372,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="329" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
         <v>483</v>
       </c>
@@ -8385,7 +8380,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="330" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
         <v>485</v>
       </c>
@@ -8393,7 +8388,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="331" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
         <v>487</v>
       </c>
@@ -8401,7 +8396,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="332" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
         <v>491</v>
       </c>
@@ -8409,7 +8404,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="333" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
         <v>493</v>
       </c>
@@ -8417,7 +8412,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="334" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
         <v>496</v>
       </c>
@@ -8425,7 +8420,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="335" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
         <v>500</v>
       </c>
@@ -8433,7 +8428,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="336" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
         <v>505</v>
       </c>
@@ -8441,7 +8436,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="337" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
         <v>507</v>
       </c>
@@ -8449,7 +8444,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="338" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
         <v>509</v>
       </c>
@@ -8457,7 +8452,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="339" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
         <v>511</v>
       </c>
@@ -8465,7 +8460,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="340" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
         <v>513</v>
       </c>
@@ -8473,7 +8468,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="341" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
         <v>515</v>
       </c>
@@ -8481,7 +8476,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="342" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
         <v>518</v>
       </c>
@@ -8489,7 +8484,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="343" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
         <v>529</v>
       </c>
@@ -8497,7 +8492,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="344" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
         <v>531</v>
       </c>
@@ -8505,7 +8500,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="345" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
         <v>533</v>
       </c>
@@ -8513,7 +8508,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="346" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
         <v>543</v>
       </c>
@@ -8521,7 +8516,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="347" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
         <v>545</v>
       </c>
@@ -8529,7 +8524,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="348" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
         <v>550</v>
       </c>
@@ -8537,7 +8532,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="349" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
         <v>555</v>
       </c>
@@ -8545,7 +8540,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="350" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
         <v>560</v>
       </c>
@@ -8553,7 +8548,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="351" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
         <v>564</v>
       </c>
@@ -8561,7 +8556,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="352" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
         <v>568</v>
       </c>
@@ -8569,7 +8564,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="353" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
         <v>570</v>
       </c>
@@ -8577,7 +8572,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="354" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
         <v>572</v>
       </c>
@@ -8585,7 +8580,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="355" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
         <v>596</v>
       </c>
@@ -8593,7 +8588,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="356" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
         <v>604</v>
       </c>
@@ -8601,7 +8596,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="357" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
         <v>609</v>
       </c>
@@ -8609,7 +8604,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="358" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
         <v>611</v>
       </c>
@@ -8617,7 +8612,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="359" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
         <v>613</v>
       </c>
@@ -8625,7 +8620,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="360" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
         <v>615</v>
       </c>
@@ -8633,7 +8628,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="361" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
         <v>617</v>
       </c>
@@ -8641,7 +8636,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="362" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
         <v>627</v>
       </c>
@@ -8649,7 +8644,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="363" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
         <v>629</v>
       </c>
@@ -8657,7 +8652,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="364" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
         <v>631</v>
       </c>
@@ -8665,7 +8660,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="365" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B365">
         <v>10195</v>
       </c>
@@ -8673,7 +8668,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="366" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B366">
         <v>10419</v>
       </c>
@@ -8681,7 +8676,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="367" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B367">
         <v>10533</v>
       </c>
@@ -8689,7 +8684,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="368" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B368">
         <v>10620</v>
       </c>
@@ -8697,7 +8692,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="369" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B369">
         <v>10626</v>
       </c>
@@ -8705,7 +8700,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="370" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="370" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B370">
         <v>10658</v>
       </c>
@@ -8713,7 +8708,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="371" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B371" s="4">
         <v>10681</v>
       </c>
@@ -8721,7 +8716,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="372" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B372">
         <v>10783</v>
       </c>
@@ -8729,7 +8724,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="373" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B373" s="4">
         <v>10835</v>
       </c>
@@ -8737,7 +8732,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="374" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="374" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B374">
         <v>10838</v>
       </c>
@@ -8745,7 +8740,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="375" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="375" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B375">
         <v>10863</v>
       </c>
@@ -8753,7 +8748,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="376" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B376" s="4">
         <v>10890</v>
       </c>
@@ -8761,7 +8756,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="377" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="377" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B377">
         <v>10900</v>
       </c>
@@ -8769,7 +8764,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="378" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="378" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B378" s="4">
         <v>10904</v>
       </c>
@@ -8777,7 +8772,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="379" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="379" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B379">
         <v>10909</v>
       </c>
@@ -8785,7 +8780,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="380" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="380" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B380">
         <v>10919</v>
       </c>
@@ -8793,7 +8788,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="381" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="381" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B381">
         <v>10920</v>
       </c>
@@ -8801,7 +8796,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="382" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B382" s="4">
         <v>10930</v>
       </c>
@@ -8809,7 +8804,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="383" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="383" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B383" s="4">
         <v>11382</v>
       </c>
@@ -8817,7 +8812,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="384" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="384" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B384">
         <v>11389</v>
       </c>
@@ -8825,7 +8820,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="385" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="385" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B385">
         <v>11513</v>
       </c>
@@ -8833,7 +8828,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="386" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="386" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B386">
         <v>11766</v>
       </c>
@@ -8841,7 +8836,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="387" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="387" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B387">
         <v>11767</v>
       </c>
@@ -8849,7 +8844,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="388" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="388" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B388" s="4">
         <v>11804</v>
       </c>
@@ -8857,7 +8852,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="389" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="389" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B389">
         <v>11827</v>
       </c>
@@ -8865,7 +8860,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="390" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="390" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B390">
         <v>11876</v>
       </c>
@@ -8873,7 +8868,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="391" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="391" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B391">
         <v>11981</v>
       </c>
@@ -8881,7 +8876,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="392" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="392" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B392">
         <v>12184</v>
       </c>
@@ -8889,7 +8884,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="393" spans="2:5" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="393" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B393" s="4">
         <v>12404</v>
       </c>
@@ -8897,7 +8892,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="394" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="394" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B394">
         <v>12466</v>
       </c>
@@ -8905,7 +8900,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="395" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="395" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B395">
         <v>12660</v>
       </c>
@@ -8913,7 +8908,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="396" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="396" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B396">
         <v>12678</v>
       </c>
@@ -8921,7 +8916,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="397" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="397" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B397">
         <v>12815</v>
       </c>
@@ -8929,7 +8924,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="398" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="398" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B398">
         <v>12841</v>
       </c>
@@ -8937,7 +8932,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="399" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="399" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B399">
         <v>10306</v>
       </c>
@@ -8945,7 +8940,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="400" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="400" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B400">
         <v>10647</v>
       </c>
@@ -8953,7 +8948,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="401" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="401" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B401">
         <v>11046</v>
       </c>
@@ -8961,7 +8956,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="402" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="402" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B402">
         <v>11103</v>
       </c>
@@ -8969,7 +8964,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="403" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="403" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B403">
         <v>11750</v>
       </c>
@@ -8977,7 +8972,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="404" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="404" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B404">
         <v>12555</v>
       </c>
@@ -8987,11 +8982,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G404" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="Thompson (T-1 and T-3)"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:G167">
       <sortCondition ref="A1:A404"/>
     </sortState>

</xml_diff>